<commit_message>
Actualizar plantillas de informes: Proctor SU19 v08, ContHumedad SU20 v07, EquiArena SU21 v08, LLP SU23 v07, GranSuelo SU24 v09
</commit_message>
<xml_diff>
--- a/app/templates/informes/ContHumedad/Template_ContHumedad.xlsx
+++ b/app/templates/informes/ContHumedad/Template_ContHumedad.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\3.0 Formatos e informes\2026\1.0 Informe de ensayo\1.1 Informe Suelo\INFORME ACREDITADO-E ISO\6.1 JUNIO INICIA 15-06-25\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\ContHumedad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3850AAE7-AD9E-4561-AE4F-6FC4E905F9F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{422D366B-0E4F-48EF-A099-1BA65A2E2032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1226,7 +1226,7 @@
     <t>- De conformidad con lo dispuesto por el artículo 1321 del Código Civil, queda establecido que en ningún caso la responsabilidad de GEOFAL S.A.C. será mayor al valor del servicio prestado.</t>
   </si>
   <si>
-    <t>Versión: 07 (15-06-2026)</t>
+    <t>Versión: 07 (11-06-2026)</t>
   </si>
 </sst>
 </file>
@@ -1259,7 +1259,7 @@
     <numFmt numFmtId="186" formatCode="000\-\ &quot;26&quot;"/>
     <numFmt numFmtId="187" formatCode="&quot;FORMATO F-LEM-P-SU-11.01&quot;"/>
   </numFmts>
-  <fonts count="82">
+  <fonts count="83">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1772,6 +1772,12 @@
       <u/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -2466,7 +2472,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="707">
+  <cellXfs count="708">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4226,44 +4232,100 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -4315,88 +4377,66 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="48" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="187" fontId="25" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -4405,28 +4445,33 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="16" fontId="16" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="2" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="2" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4452,15 +4497,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="2" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="2" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="38" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
@@ -4481,72 +4517,63 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="16" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="187" fontId="25" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="12" fontId="23" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="42" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="184" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -4568,9 +4595,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4588,19 +4612,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="12" fontId="23" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4638,13 +4657,28 @@
     <xf numFmtId="167" fontId="5" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="59" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="59" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="2" borderId="10" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="4" fillId="2" borderId="12" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="64" fillId="2" borderId="4" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4733,30 +4767,6 @@
     <xf numFmtId="2" fontId="16" fillId="2" borderId="40" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="62" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="59" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="59" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="2" borderId="10" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="4" fillId="2" borderId="12" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="65" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4778,8 +4788,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="82" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -5026,7 +5036,7 @@
                 <a:cs typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="77591296"/>
@@ -5062,7 +5072,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="77557120"/>
@@ -5100,7 +5110,7 @@
           <a:cs typeface="Calibri"/>
         </a:defRPr>
       </a:pPr>
-      <a:endParaRPr lang="es-ES"/>
+      <a:endParaRPr lang="es-PE"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -6523,7 +6533,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -6582,7 +6592,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="datos de ecuacion del anillo"/>
@@ -6701,7 +6711,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -6752,7 +6762,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -6804,7 +6814,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="BGA"/>
@@ -6836,7 +6846,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink6.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -7631,35 +7641,35 @@
       <c r="K6" s="16"/>
     </row>
     <row r="7" spans="1:18" ht="15.9" customHeight="1">
-      <c r="A7" s="567" t="s">
+      <c r="A7" s="544" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="567"/>
-      <c r="C7" s="567"/>
-      <c r="D7" s="567"/>
-      <c r="E7" s="567"/>
-      <c r="F7" s="567"/>
-      <c r="G7" s="567"/>
-      <c r="H7" s="567"/>
-      <c r="I7" s="567"/>
-      <c r="J7" s="567"/>
-      <c r="K7" s="567"/>
+      <c r="B7" s="544"/>
+      <c r="C7" s="544"/>
+      <c r="D7" s="544"/>
+      <c r="E7" s="544"/>
+      <c r="F7" s="544"/>
+      <c r="G7" s="544"/>
+      <c r="H7" s="544"/>
+      <c r="I7" s="544"/>
+      <c r="J7" s="544"/>
+      <c r="K7" s="544"/>
     </row>
     <row r="8" spans="1:18" ht="15.9" customHeight="1">
-      <c r="A8" s="587">
+      <c r="A8" s="565">
         <f>K13</f>
         <v>15</v>
       </c>
-      <c r="B8" s="587"/>
-      <c r="C8" s="587"/>
-      <c r="D8" s="587"/>
-      <c r="E8" s="587"/>
-      <c r="F8" s="587"/>
-      <c r="G8" s="587"/>
-      <c r="H8" s="587"/>
-      <c r="I8" s="587"/>
-      <c r="J8" s="587"/>
-      <c r="K8" s="587"/>
+      <c r="B8" s="565"/>
+      <c r="C8" s="565"/>
+      <c r="D8" s="565"/>
+      <c r="E8" s="565"/>
+      <c r="F8" s="565"/>
+      <c r="G8" s="565"/>
+      <c r="H8" s="565"/>
+      <c r="I8" s="565"/>
+      <c r="J8" s="565"/>
+      <c r="K8" s="565"/>
     </row>
     <row r="9" spans="1:18" ht="15.9" customHeight="1">
       <c r="P9" s="17"/>
@@ -7770,8 +7780,8 @@
       <c r="L13" s="25"/>
       <c r="M13" s="25"/>
       <c r="N13" s="25"/>
-      <c r="Q13" s="578"/>
-      <c r="R13" s="578"/>
+      <c r="Q13" s="556"/>
+      <c r="R13" s="556"/>
     </row>
     <row r="14" spans="1:18" ht="15.9" customHeight="1">
       <c r="A14" s="167" t="s">
@@ -7794,19 +7804,19 @@
       <c r="R14" s="304"/>
     </row>
     <row r="15" spans="1:18" ht="18" customHeight="1">
-      <c r="A15" s="579" t="s">
+      <c r="A15" s="557" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="580"/>
-      <c r="C15" s="580"/>
-      <c r="D15" s="580"/>
-      <c r="E15" s="580"/>
-      <c r="F15" s="580"/>
-      <c r="G15" s="580"/>
-      <c r="H15" s="580"/>
-      <c r="I15" s="580"/>
-      <c r="J15" s="580"/>
-      <c r="K15" s="581"/>
+      <c r="B15" s="558"/>
+      <c r="C15" s="558"/>
+      <c r="D15" s="558"/>
+      <c r="E15" s="558"/>
+      <c r="F15" s="558"/>
+      <c r="G15" s="558"/>
+      <c r="H15" s="558"/>
+      <c r="I15" s="558"/>
+      <c r="J15" s="558"/>
+      <c r="K15" s="559"/>
       <c r="L15" s="25"/>
       <c r="M15" s="25"/>
       <c r="N15" s="25"/>
@@ -7814,19 +7824,19 @@
       <c r="R15" s="304"/>
     </row>
     <row r="16" spans="1:18" ht="18" customHeight="1">
-      <c r="A16" s="584" t="s">
+      <c r="A16" s="562" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="585"/>
-      <c r="C16" s="585"/>
-      <c r="D16" s="585"/>
-      <c r="E16" s="585"/>
-      <c r="F16" s="585"/>
-      <c r="G16" s="585"/>
-      <c r="H16" s="585"/>
-      <c r="I16" s="585"/>
-      <c r="J16" s="585"/>
-      <c r="K16" s="586"/>
+      <c r="B16" s="563"/>
+      <c r="C16" s="563"/>
+      <c r="D16" s="563"/>
+      <c r="E16" s="563"/>
+      <c r="F16" s="563"/>
+      <c r="G16" s="563"/>
+      <c r="H16" s="563"/>
+      <c r="I16" s="563"/>
+      <c r="J16" s="563"/>
+      <c r="K16" s="564"/>
       <c r="L16" s="25"/>
       <c r="M16" s="25"/>
       <c r="N16" s="25"/>
@@ -7834,10 +7844,10 @@
       <c r="R16" s="304"/>
     </row>
     <row r="17" spans="1:26" ht="11.25" customHeight="1">
-      <c r="A17" s="568" t="s">
+      <c r="A17" s="545" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="569"/>
+      <c r="B17" s="546"/>
       <c r="C17" s="36"/>
       <c r="D17" s="36"/>
       <c r="E17" s="36"/>
@@ -7854,8 +7864,8 @@
       <c r="R17" s="304"/>
     </row>
     <row r="18" spans="1:26" ht="15.9" customHeight="1">
-      <c r="A18" s="570"/>
-      <c r="B18" s="571"/>
+      <c r="A18" s="547"/>
+      <c r="B18" s="548"/>
       <c r="C18" s="39"/>
       <c r="D18" s="39"/>
       <c r="E18" s="39"/>
@@ -8000,10 +8010,10 @@
       <c r="P21" s="93" t="s">
         <v>32</v>
       </c>
-      <c r="Q21" s="550">
+      <c r="Q21" s="588">
         <v>44090</v>
       </c>
-      <c r="R21" s="550"/>
+      <c r="R21" s="588"/>
       <c r="S21" s="94"/>
       <c r="T21" s="95"/>
       <c r="U21" s="94"/>
@@ -8046,15 +8056,15 @@
     </row>
     <row r="23" spans="1:26" ht="13.5" customHeight="1" thickBot="1">
       <c r="A23" s="168"/>
-      <c r="B23" s="588"/>
-      <c r="C23" s="588"/>
+      <c r="B23" s="566"/>
+      <c r="C23" s="566"/>
       <c r="D23" s="306"/>
       <c r="E23" s="306"/>
       <c r="F23" s="306"/>
       <c r="G23" s="306"/>
       <c r="H23" s="306"/>
-      <c r="I23" s="588"/>
-      <c r="J23" s="588"/>
+      <c r="I23" s="566"/>
+      <c r="J23" s="566"/>
       <c r="K23" s="168"/>
       <c r="L23" s="25"/>
       <c r="M23" s="49"/>
@@ -8076,8 +8086,8 @@
         <f>+R24</f>
         <v>1</v>
       </c>
-      <c r="I24" s="582"/>
-      <c r="J24" s="582"/>
+      <c r="I24" s="560"/>
+      <c r="J24" s="560"/>
       <c r="K24" s="305"/>
       <c r="L24" s="25"/>
       <c r="M24" s="54"/>
@@ -8091,21 +8101,21 @@
       <c r="R24" s="56">
         <v>1</v>
       </c>
-      <c r="S24" s="551" t="s">
+      <c r="S24" s="549" t="s">
         <v>37</v>
       </c>
       <c r="U24" s="56">
         <v>2</v>
       </c>
-      <c r="V24" s="551" t="s">
+      <c r="V24" s="549" t="s">
         <v>37</v>
       </c>
-      <c r="W24" s="546" t="s">
+      <c r="W24" s="584" t="s">
         <v>38</v>
       </c>
-      <c r="X24" s="546"/>
-      <c r="Y24" s="546"/>
-      <c r="Z24" s="547"/>
+      <c r="X24" s="584"/>
+      <c r="Y24" s="584"/>
+      <c r="Z24" s="585"/>
     </row>
     <row r="25" spans="1:26" ht="17.25" customHeight="1" thickBot="1">
       <c r="A25" s="171"/>
@@ -8123,8 +8133,8 @@
         <f>+R25</f>
         <v>1</v>
       </c>
-      <c r="I25" s="582"/>
-      <c r="J25" s="582"/>
+      <c r="I25" s="560"/>
+      <c r="J25" s="560"/>
       <c r="K25" s="305"/>
       <c r="L25" s="25"/>
       <c r="M25" s="54"/>
@@ -8138,15 +8148,15 @@
       <c r="R25" s="59">
         <v>1</v>
       </c>
-      <c r="S25" s="551"/>
+      <c r="S25" s="549"/>
       <c r="U25" s="59">
         <v>2</v>
       </c>
-      <c r="V25" s="551"/>
-      <c r="W25" s="548"/>
-      <c r="X25" s="548"/>
-      <c r="Y25" s="548"/>
-      <c r="Z25" s="549"/>
+      <c r="V25" s="549"/>
+      <c r="W25" s="586"/>
+      <c r="X25" s="586"/>
+      <c r="Y25" s="586"/>
+      <c r="Z25" s="587"/>
     </row>
     <row r="26" spans="1:26" ht="17.25" customHeight="1">
       <c r="A26" s="171"/>
@@ -8164,8 +8174,8 @@
         <f>S26</f>
         <v>794.6995891401001</v>
       </c>
-      <c r="I26" s="583"/>
-      <c r="J26" s="583"/>
+      <c r="I26" s="561"/>
+      <c r="J26" s="561"/>
       <c r="K26" s="169"/>
       <c r="L26" s="60"/>
       <c r="M26" s="54"/>
@@ -8507,14 +8517,14 @@
       <c r="L34" s="25"/>
       <c r="M34" s="25"/>
       <c r="N34" s="25"/>
-      <c r="P34" s="572" t="s">
+      <c r="P34" s="550" t="s">
         <v>59</v>
       </c>
-      <c r="Q34" s="573"/>
-      <c r="R34" s="576" t="s">
+      <c r="Q34" s="551"/>
+      <c r="R34" s="554" t="s">
         <v>60</v>
       </c>
-      <c r="S34" s="576" t="s">
+      <c r="S34" s="554" t="s">
         <v>61</v>
       </c>
       <c r="T34" s="132"/>
@@ -8527,10 +8537,10 @@
       <c r="L35" s="25"/>
       <c r="M35" s="25"/>
       <c r="N35" s="25"/>
-      <c r="P35" s="574"/>
-      <c r="Q35" s="575"/>
-      <c r="R35" s="577"/>
-      <c r="S35" s="577"/>
+      <c r="P35" s="552"/>
+      <c r="Q35" s="553"/>
+      <c r="R35" s="555"/>
+      <c r="S35" s="555"/>
       <c r="T35" s="133"/>
       <c r="U35" s="132"/>
       <c r="V35" s="132"/>
@@ -8618,7 +8628,7 @@
       <c r="L38" s="25"/>
       <c r="M38" s="25"/>
       <c r="N38" s="25"/>
-      <c r="P38" s="554" t="s">
+      <c r="P38" s="570" t="s">
         <v>72</v>
       </c>
       <c r="Q38" s="108">
@@ -8635,16 +8645,16 @@
       <c r="V38" s="135"/>
     </row>
     <row r="39" spans="1:22" ht="14.25" customHeight="1">
-      <c r="A39" s="552" t="s">
+      <c r="A39" s="567" t="s">
         <v>75</v>
       </c>
-      <c r="B39" s="552"/>
-      <c r="C39" s="552"/>
-      <c r="D39" s="552"/>
-      <c r="E39" s="552"/>
-      <c r="F39" s="552"/>
-      <c r="G39" s="552"/>
-      <c r="H39" s="553"/>
+      <c r="B39" s="567"/>
+      <c r="C39" s="567"/>
+      <c r="D39" s="567"/>
+      <c r="E39" s="567"/>
+      <c r="F39" s="567"/>
+      <c r="G39" s="567"/>
+      <c r="H39" s="568"/>
       <c r="I39" s="166" t="s">
         <v>67</v>
       </c>
@@ -8653,7 +8663,7 @@
       <c r="L39" s="25"/>
       <c r="M39" s="25"/>
       <c r="N39" s="25"/>
-      <c r="P39" s="555"/>
+      <c r="P39" s="571"/>
       <c r="Q39" s="108">
         <v>0.75</v>
       </c>
@@ -8678,7 +8688,7 @@
       <c r="L40" s="25"/>
       <c r="M40" s="25"/>
       <c r="N40" s="25"/>
-      <c r="P40" s="555"/>
+      <c r="P40" s="571"/>
       <c r="Q40" s="108">
         <v>1.5</v>
       </c>
@@ -8705,7 +8715,7 @@
       <c r="L41" s="25"/>
       <c r="M41" s="25"/>
       <c r="N41" s="25"/>
-      <c r="P41" s="556"/>
+      <c r="P41" s="572"/>
       <c r="Q41" s="104">
         <v>3</v>
       </c>
@@ -8836,7 +8846,7 @@
       </c>
       <c r="T45" s="86"/>
       <c r="U45" s="102"/>
-      <c r="V45" s="545"/>
+      <c r="V45" s="569"/>
     </row>
     <row r="46" spans="1:22" ht="15.9" customHeight="1">
       <c r="C46" s="42"/>
@@ -8862,7 +8872,7 @@
       </c>
       <c r="T46" s="86"/>
       <c r="U46" s="106"/>
-      <c r="V46" s="545"/>
+      <c r="V46" s="569"/>
     </row>
     <row r="47" spans="1:22" ht="12.75" customHeight="1">
       <c r="A47" s="154" t="s">
@@ -8951,30 +8961,30 @@
       <c r="V50" s="107"/>
     </row>
     <row r="51" spans="1:22" ht="33" customHeight="1">
-      <c r="A51" s="566" t="s">
+      <c r="A51" s="582" t="s">
         <v>96</v>
       </c>
-      <c r="B51" s="566"/>
-      <c r="C51" s="566"/>
-      <c r="D51" s="566"/>
-      <c r="E51" s="566"/>
-      <c r="F51" s="566"/>
-      <c r="G51" s="566"/>
-      <c r="H51" s="566"/>
-      <c r="I51" s="566"/>
-      <c r="J51" s="566"/>
-      <c r="K51" s="566"/>
+      <c r="B51" s="582"/>
+      <c r="C51" s="582"/>
+      <c r="D51" s="582"/>
+      <c r="E51" s="582"/>
+      <c r="F51" s="582"/>
+      <c r="G51" s="582"/>
+      <c r="H51" s="582"/>
+      <c r="I51" s="582"/>
+      <c r="J51" s="582"/>
+      <c r="K51" s="582"/>
       <c r="T51" s="86"/>
       <c r="U51" s="109"/>
       <c r="V51" s="107"/>
     </row>
     <row r="52" spans="1:22" ht="11.25" customHeight="1">
-      <c r="H52" s="565" t="s">
+      <c r="H52" s="581" t="s">
         <v>97</v>
       </c>
-      <c r="I52" s="565"/>
-      <c r="J52" s="565"/>
-      <c r="K52" s="565"/>
+      <c r="I52" s="581"/>
+      <c r="J52" s="581"/>
+      <c r="K52" s="581"/>
       <c r="T52" s="86"/>
       <c r="U52" s="109"/>
       <c r="V52" s="107"/>
@@ -8989,14 +8999,14 @@
     <row r="54" spans="1:22">
       <c r="J54" s="72"/>
       <c r="K54" s="71"/>
-      <c r="T54" s="544"/>
+      <c r="T54" s="583"/>
       <c r="U54" s="109"/>
       <c r="V54" s="107"/>
     </row>
     <row r="55" spans="1:22">
       <c r="J55"/>
       <c r="K55" s="71"/>
-      <c r="T55" s="544"/>
+      <c r="T55" s="583"/>
       <c r="U55" s="109"/>
       <c r="V55" s="107"/>
     </row>
@@ -9036,58 +9046,58 @@
       <c r="K58" s="73"/>
     </row>
     <row r="59" spans="1:22">
-      <c r="A59" s="557" t="s">
+      <c r="A59" s="573" t="s">
         <v>98</v>
       </c>
-      <c r="B59" s="559"/>
-      <c r="C59" s="559"/>
-      <c r="D59" s="559"/>
-      <c r="E59" s="559"/>
-      <c r="F59" s="559"/>
-      <c r="G59" s="559"/>
-      <c r="H59" s="559"/>
-      <c r="I59" s="559"/>
-      <c r="J59" s="559"/>
-      <c r="K59" s="560"/>
+      <c r="B59" s="575"/>
+      <c r="C59" s="575"/>
+      <c r="D59" s="575"/>
+      <c r="E59" s="575"/>
+      <c r="F59" s="575"/>
+      <c r="G59" s="575"/>
+      <c r="H59" s="575"/>
+      <c r="I59" s="575"/>
+      <c r="J59" s="575"/>
+      <c r="K59" s="576"/>
     </row>
     <row r="60" spans="1:22">
-      <c r="A60" s="558"/>
-      <c r="B60" s="561"/>
-      <c r="C60" s="561"/>
-      <c r="D60" s="561"/>
-      <c r="E60" s="561"/>
-      <c r="F60" s="561"/>
-      <c r="G60" s="561"/>
-      <c r="H60" s="561"/>
-      <c r="I60" s="561"/>
-      <c r="J60" s="561"/>
-      <c r="K60" s="562"/>
+      <c r="A60" s="574"/>
+      <c r="B60" s="577"/>
+      <c r="C60" s="577"/>
+      <c r="D60" s="577"/>
+      <c r="E60" s="577"/>
+      <c r="F60" s="577"/>
+      <c r="G60" s="577"/>
+      <c r="H60" s="577"/>
+      <c r="I60" s="577"/>
+      <c r="J60" s="577"/>
+      <c r="K60" s="578"/>
     </row>
     <row r="61" spans="1:22">
       <c r="A61" s="74"/>
-      <c r="B61" s="561"/>
-      <c r="C61" s="561"/>
-      <c r="D61" s="561"/>
-      <c r="E61" s="561"/>
-      <c r="F61" s="561"/>
-      <c r="G61" s="561"/>
-      <c r="H61" s="561"/>
-      <c r="I61" s="561"/>
-      <c r="J61" s="561"/>
-      <c r="K61" s="562"/>
+      <c r="B61" s="577"/>
+      <c r="C61" s="577"/>
+      <c r="D61" s="577"/>
+      <c r="E61" s="577"/>
+      <c r="F61" s="577"/>
+      <c r="G61" s="577"/>
+      <c r="H61" s="577"/>
+      <c r="I61" s="577"/>
+      <c r="J61" s="577"/>
+      <c r="K61" s="578"/>
     </row>
     <row r="62" spans="1:22">
       <c r="A62" s="75"/>
-      <c r="B62" s="563"/>
-      <c r="C62" s="563"/>
-      <c r="D62" s="563"/>
-      <c r="E62" s="563"/>
-      <c r="F62" s="563"/>
-      <c r="G62" s="563"/>
-      <c r="H62" s="563"/>
-      <c r="I62" s="563"/>
-      <c r="J62" s="563"/>
-      <c r="K62" s="564"/>
+      <c r="B62" s="579"/>
+      <c r="C62" s="579"/>
+      <c r="D62" s="579"/>
+      <c r="E62" s="579"/>
+      <c r="F62" s="579"/>
+      <c r="G62" s="579"/>
+      <c r="H62" s="579"/>
+      <c r="I62" s="579"/>
+      <c r="J62" s="579"/>
+      <c r="K62" s="580"/>
     </row>
     <row r="63" spans="1:22">
       <c r="A63" s="76"/>
@@ -9183,15 +9193,15 @@
       <c r="K85"/>
     </row>
     <row r="86" spans="8:11">
-      <c r="H86" s="545"/>
-      <c r="I86" s="545"/>
-      <c r="J86" s="545"/>
+      <c r="H86" s="569"/>
+      <c r="I86" s="569"/>
+      <c r="J86" s="569"/>
       <c r="K86"/>
     </row>
     <row r="87" spans="8:11">
-      <c r="H87" s="545"/>
-      <c r="I87" s="545"/>
-      <c r="J87" s="545"/>
+      <c r="H87" s="569"/>
+      <c r="I87" s="569"/>
+      <c r="J87" s="569"/>
       <c r="K87"/>
     </row>
     <row r="88" spans="8:11">
@@ -9305,6 +9315,20 @@
     <protectedRange sqref="C10:C11" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="29">
+    <mergeCell ref="T54:T55"/>
+    <mergeCell ref="V45:V46"/>
+    <mergeCell ref="W24:Z25"/>
+    <mergeCell ref="Q21:R21"/>
+    <mergeCell ref="S24:S25"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="H86:H87"/>
+    <mergeCell ref="I86:I87"/>
+    <mergeCell ref="J86:J87"/>
+    <mergeCell ref="P38:P41"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="B59:K62"/>
+    <mergeCell ref="H52:K52"/>
+    <mergeCell ref="A51:K51"/>
     <mergeCell ref="A7:K7"/>
     <mergeCell ref="A17:B18"/>
     <mergeCell ref="V24:V25"/>
@@ -9320,20 +9344,6 @@
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="I23:J23"/>
     <mergeCell ref="I24:J24"/>
-    <mergeCell ref="A39:H39"/>
-    <mergeCell ref="H86:H87"/>
-    <mergeCell ref="I86:I87"/>
-    <mergeCell ref="J86:J87"/>
-    <mergeCell ref="P38:P41"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="B59:K62"/>
-    <mergeCell ref="H52:K52"/>
-    <mergeCell ref="A51:K51"/>
-    <mergeCell ref="T54:T55"/>
-    <mergeCell ref="V45:V46"/>
-    <mergeCell ref="W24:Z25"/>
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="S24:S25"/>
   </mergeCells>
   <conditionalFormatting sqref="A39">
     <cfRule type="cellIs" priority="1" stopIfTrue="1" operator="between">
@@ -9472,40 +9482,40 @@
       <c r="P6" s="454"/>
     </row>
     <row r="7" spans="1:16" ht="15.9" customHeight="1">
-      <c r="A7" s="620" t="s">
+      <c r="A7" s="591" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="620"/>
-      <c r="C7" s="620"/>
-      <c r="D7" s="620"/>
-      <c r="E7" s="620"/>
-      <c r="F7" s="620"/>
-      <c r="G7" s="620"/>
-      <c r="H7" s="620"/>
-      <c r="I7" s="620"/>
-      <c r="J7" s="620"/>
-      <c r="K7" s="620"/>
-      <c r="L7" s="620"/>
+      <c r="B7" s="591"/>
+      <c r="C7" s="591"/>
+      <c r="D7" s="591"/>
+      <c r="E7" s="591"/>
+      <c r="F7" s="591"/>
+      <c r="G7" s="591"/>
+      <c r="H7" s="591"/>
+      <c r="I7" s="591"/>
+      <c r="J7" s="591"/>
+      <c r="K7" s="591"/>
+      <c r="L7" s="591"/>
       <c r="O7" s="450" t="s">
         <v>233</v>
       </c>
       <c r="P7" s="454"/>
     </row>
     <row r="8" spans="1:16" ht="15.9" customHeight="1">
-      <c r="A8" s="621" t="s">
+      <c r="A8" s="592" t="s">
         <v>250</v>
       </c>
-      <c r="B8" s="621"/>
-      <c r="C8" s="621"/>
-      <c r="D8" s="621"/>
-      <c r="E8" s="621"/>
-      <c r="F8" s="621"/>
-      <c r="G8" s="621"/>
-      <c r="H8" s="621"/>
-      <c r="I8" s="621"/>
-      <c r="J8" s="621"/>
-      <c r="K8" s="621"/>
-      <c r="L8" s="621"/>
+      <c r="B8" s="592"/>
+      <c r="C8" s="592"/>
+      <c r="D8" s="592"/>
+      <c r="E8" s="592"/>
+      <c r="F8" s="592"/>
+      <c r="G8" s="592"/>
+      <c r="H8" s="592"/>
+      <c r="I8" s="592"/>
+      <c r="J8" s="592"/>
+      <c r="K8" s="592"/>
+      <c r="L8" s="592"/>
       <c r="O8" s="450" t="s">
         <v>296</v>
       </c>
@@ -9604,39 +9614,39 @@
       <c r="P13" s="455"/>
     </row>
     <row r="14" spans="1:16" ht="17.25" customHeight="1">
-      <c r="A14" s="622" t="s">
+      <c r="A14" s="593" t="s">
         <v>102</v>
       </c>
-      <c r="B14" s="623"/>
-      <c r="C14" s="623"/>
-      <c r="D14" s="623"/>
-      <c r="E14" s="623"/>
-      <c r="F14" s="623"/>
-      <c r="G14" s="623"/>
-      <c r="H14" s="623"/>
-      <c r="I14" s="623"/>
-      <c r="J14" s="623"/>
-      <c r="K14" s="623"/>
-      <c r="L14" s="624"/>
+      <c r="B14" s="594"/>
+      <c r="C14" s="594"/>
+      <c r="D14" s="594"/>
+      <c r="E14" s="594"/>
+      <c r="F14" s="594"/>
+      <c r="G14" s="594"/>
+      <c r="H14" s="594"/>
+      <c r="I14" s="594"/>
+      <c r="J14" s="594"/>
+      <c r="K14" s="594"/>
+      <c r="L14" s="595"/>
       <c r="M14" s="87"/>
       <c r="O14" s="453"/>
       <c r="P14" s="454"/>
     </row>
     <row r="15" spans="1:16" ht="15" customHeight="1">
-      <c r="A15" s="625" t="s">
+      <c r="A15" s="596" t="s">
         <v>103</v>
       </c>
-      <c r="B15" s="626"/>
-      <c r="C15" s="626"/>
-      <c r="D15" s="626"/>
-      <c r="E15" s="626"/>
-      <c r="F15" s="626"/>
-      <c r="G15" s="626"/>
-      <c r="H15" s="626"/>
-      <c r="I15" s="626"/>
-      <c r="J15" s="626"/>
-      <c r="K15" s="626"/>
-      <c r="L15" s="627"/>
+      <c r="B15" s="597"/>
+      <c r="C15" s="597"/>
+      <c r="D15" s="597"/>
+      <c r="E15" s="597"/>
+      <c r="F15" s="597"/>
+      <c r="G15" s="597"/>
+      <c r="H15" s="597"/>
+      <c r="I15" s="597"/>
+      <c r="J15" s="597"/>
+      <c r="K15" s="597"/>
+      <c r="L15" s="598"/>
       <c r="M15" s="87"/>
       <c r="O15" s="450" t="s">
         <v>104</v>
@@ -9663,17 +9673,17 @@
       <c r="P16" s="456"/>
     </row>
     <row r="17" spans="1:19" ht="15.9" customHeight="1">
-      <c r="A17" s="618" t="s">
+      <c r="A17" s="589" t="s">
         <v>254</v>
       </c>
-      <c r="B17" s="619"/>
-      <c r="C17" s="619"/>
-      <c r="D17" s="619"/>
-      <c r="E17" s="619"/>
-      <c r="F17" s="619"/>
-      <c r="G17" s="619"/>
-      <c r="H17" s="619"/>
-      <c r="I17" s="619"/>
+      <c r="B17" s="590"/>
+      <c r="C17" s="590"/>
+      <c r="D17" s="590"/>
+      <c r="E17" s="590"/>
+      <c r="F17" s="590"/>
+      <c r="G17" s="590"/>
+      <c r="H17" s="590"/>
+      <c r="I17" s="590"/>
       <c r="J17" s="431"/>
       <c r="K17" s="431"/>
       <c r="L17" s="487"/>
@@ -9777,12 +9787,12 @@
       <c r="L23" s="487"/>
     </row>
     <row r="24" spans="1:19" ht="15.9" customHeight="1">
-      <c r="A24" s="618" t="s">
+      <c r="A24" s="589" t="s">
         <v>256</v>
       </c>
-      <c r="B24" s="619"/>
-      <c r="C24" s="619"/>
-      <c r="D24" s="619"/>
+      <c r="B24" s="590"/>
+      <c r="C24" s="590"/>
+      <c r="D24" s="590"/>
       <c r="E24" s="432"/>
       <c r="F24" s="432"/>
       <c r="G24" s="432"/>
@@ -9793,50 +9803,50 @@
       <c r="L24" s="487"/>
     </row>
     <row r="25" spans="1:19" ht="19.2" customHeight="1">
-      <c r="A25" s="590" t="s">
+      <c r="A25" s="599" t="s">
         <v>257</v>
       </c>
-      <c r="B25" s="590"/>
-      <c r="C25" s="590"/>
-      <c r="D25" s="590"/>
-      <c r="E25" s="591"/>
-      <c r="F25" s="591"/>
+      <c r="B25" s="599"/>
+      <c r="C25" s="599"/>
+      <c r="D25" s="599"/>
+      <c r="E25" s="600"/>
+      <c r="F25" s="600"/>
       <c r="G25" s="433"/>
-      <c r="H25" s="614" t="s">
+      <c r="H25" s="601" t="s">
         <v>286</v>
       </c>
-      <c r="I25" s="615"/>
-      <c r="J25" s="616"/>
+      <c r="I25" s="602"/>
+      <c r="J25" s="603"/>
       <c r="K25" s="493"/>
       <c r="L25" s="487"/>
     </row>
     <row r="26" spans="1:19" ht="19.2" customHeight="1">
-      <c r="A26" s="590" t="s">
+      <c r="A26" s="599" t="s">
         <v>258</v>
       </c>
-      <c r="B26" s="590"/>
-      <c r="C26" s="590"/>
-      <c r="D26" s="590"/>
-      <c r="E26" s="591"/>
-      <c r="F26" s="591"/>
+      <c r="B26" s="599"/>
+      <c r="C26" s="599"/>
+      <c r="D26" s="599"/>
+      <c r="E26" s="600"/>
+      <c r="F26" s="600"/>
       <c r="G26" s="433"/>
-      <c r="H26" s="617" t="s">
+      <c r="H26" s="604" t="s">
         <v>287</v>
       </c>
-      <c r="I26" s="617"/>
+      <c r="I26" s="604"/>
       <c r="J26" s="434"/>
       <c r="K26" s="494"/>
       <c r="L26" s="487"/>
     </row>
     <row r="27" spans="1:19" ht="19.2" customHeight="1">
-      <c r="A27" s="590" t="s">
+      <c r="A27" s="599" t="s">
         <v>259</v>
       </c>
-      <c r="B27" s="590"/>
-      <c r="C27" s="590"/>
-      <c r="D27" s="590"/>
-      <c r="E27" s="591"/>
-      <c r="F27" s="591"/>
+      <c r="B27" s="599"/>
+      <c r="C27" s="599"/>
+      <c r="D27" s="599"/>
+      <c r="E27" s="600"/>
+      <c r="F27" s="600"/>
       <c r="G27" s="433"/>
       <c r="H27" s="446"/>
       <c r="I27" s="447"/>
@@ -9846,14 +9856,14 @@
       <c r="M27" s="87"/>
     </row>
     <row r="28" spans="1:19" ht="19.2" customHeight="1">
-      <c r="A28" s="590" t="s">
+      <c r="A28" s="599" t="s">
         <v>288</v>
       </c>
-      <c r="B28" s="590"/>
-      <c r="C28" s="590"/>
-      <c r="D28" s="590"/>
-      <c r="E28" s="591"/>
-      <c r="F28" s="591"/>
+      <c r="B28" s="599"/>
+      <c r="C28" s="599"/>
+      <c r="D28" s="599"/>
+      <c r="E28" s="600"/>
+      <c r="F28" s="600"/>
       <c r="L28" s="495"/>
       <c r="M28" s="87"/>
     </row>
@@ -9874,22 +9884,22 @@
     </row>
     <row r="30" spans="1:19" ht="15.75" customHeight="1">
       <c r="A30" s="501"/>
-      <c r="B30" s="612" t="s">
+      <c r="B30" s="608" t="s">
         <v>261</v>
       </c>
-      <c r="C30" s="612"/>
-      <c r="D30" s="612"/>
-      <c r="E30" s="612"/>
-      <c r="F30" s="612"/>
-      <c r="G30" s="612"/>
+      <c r="C30" s="608"/>
+      <c r="D30" s="608"/>
+      <c r="E30" s="608"/>
+      <c r="F30" s="608"/>
+      <c r="G30" s="608"/>
       <c r="H30" s="502" t="s">
         <v>262</v>
       </c>
       <c r="I30" s="502" t="s">
         <v>263</v>
       </c>
-      <c r="J30" s="613"/>
-      <c r="K30" s="613"/>
+      <c r="J30" s="609"/>
+      <c r="K30" s="609"/>
       <c r="L30" s="503"/>
       <c r="M30" s="87"/>
     </row>
@@ -9898,13 +9908,13 @@
       <c r="B31" s="505">
         <v>1</v>
       </c>
-      <c r="C31" s="604" t="s">
+      <c r="C31" s="605" t="s">
         <v>35</v>
       </c>
-      <c r="D31" s="605"/>
-      <c r="E31" s="605"/>
-      <c r="F31" s="605"/>
-      <c r="G31" s="606"/>
+      <c r="D31" s="606"/>
+      <c r="E31" s="606"/>
+      <c r="F31" s="606"/>
+      <c r="G31" s="607"/>
       <c r="H31" s="506" t="s">
         <v>36</v>
       </c>
@@ -9919,13 +9929,13 @@
       <c r="B32" s="510">
         <v>2</v>
       </c>
-      <c r="C32" s="604" t="s">
+      <c r="C32" s="605" t="s">
         <v>111</v>
       </c>
-      <c r="D32" s="605"/>
-      <c r="E32" s="605"/>
-      <c r="F32" s="605"/>
-      <c r="G32" s="606"/>
+      <c r="D32" s="606"/>
+      <c r="E32" s="606"/>
+      <c r="F32" s="606"/>
+      <c r="G32" s="607"/>
       <c r="H32" s="506" t="s">
         <v>36</v>
       </c>
@@ -9941,13 +9951,13 @@
       <c r="B33" s="510">
         <v>3</v>
       </c>
-      <c r="C33" s="604" t="s">
+      <c r="C33" s="605" t="s">
         <v>112</v>
       </c>
-      <c r="D33" s="605"/>
-      <c r="E33" s="605"/>
-      <c r="F33" s="605"/>
-      <c r="G33" s="606"/>
+      <c r="D33" s="606"/>
+      <c r="E33" s="606"/>
+      <c r="F33" s="606"/>
+      <c r="G33" s="607"/>
       <c r="H33" s="506" t="s">
         <v>184</v>
       </c>
@@ -9963,13 +9973,13 @@
       <c r="B34" s="505">
         <v>4</v>
       </c>
-      <c r="C34" s="604" t="s">
+      <c r="C34" s="605" t="s">
         <v>113</v>
       </c>
-      <c r="D34" s="605"/>
-      <c r="E34" s="605"/>
-      <c r="F34" s="605"/>
-      <c r="G34" s="606"/>
+      <c r="D34" s="606"/>
+      <c r="E34" s="606"/>
+      <c r="F34" s="606"/>
+      <c r="G34" s="607"/>
       <c r="H34" s="506" t="s">
         <v>184</v>
       </c>
@@ -9987,13 +9997,13 @@
       <c r="B35" s="510">
         <v>5</v>
       </c>
-      <c r="C35" s="604" t="s">
+      <c r="C35" s="605" t="s">
         <v>265</v>
       </c>
-      <c r="D35" s="605"/>
-      <c r="E35" s="605"/>
-      <c r="F35" s="605"/>
-      <c r="G35" s="606"/>
+      <c r="D35" s="606"/>
+      <c r="E35" s="606"/>
+      <c r="F35" s="606"/>
+      <c r="G35" s="607"/>
       <c r="H35" s="506" t="s">
         <v>184</v>
       </c>
@@ -10011,13 +10021,13 @@
       <c r="B36" s="505">
         <v>6</v>
       </c>
-      <c r="C36" s="604" t="s">
+      <c r="C36" s="605" t="s">
         <v>114</v>
       </c>
-      <c r="D36" s="605"/>
-      <c r="E36" s="605"/>
-      <c r="F36" s="605"/>
-      <c r="G36" s="606"/>
+      <c r="D36" s="606"/>
+      <c r="E36" s="606"/>
+      <c r="F36" s="606"/>
+      <c r="G36" s="607"/>
       <c r="H36" s="506" t="s">
         <v>184</v>
       </c>
@@ -10035,13 +10045,13 @@
       <c r="B37" s="510">
         <v>7</v>
       </c>
-      <c r="C37" s="604" t="s">
+      <c r="C37" s="605" t="s">
         <v>294</v>
       </c>
-      <c r="D37" s="605"/>
-      <c r="E37" s="605"/>
-      <c r="F37" s="605"/>
-      <c r="G37" s="606"/>
+      <c r="D37" s="606"/>
+      <c r="E37" s="606"/>
+      <c r="F37" s="606"/>
+      <c r="G37" s="607"/>
       <c r="H37" s="506" t="s">
         <v>184</v>
       </c>
@@ -10059,13 +10069,13 @@
       <c r="B38" s="510">
         <v>8</v>
       </c>
-      <c r="C38" s="604" t="s">
+      <c r="C38" s="605" t="s">
         <v>266</v>
       </c>
-      <c r="D38" s="605"/>
-      <c r="E38" s="605"/>
-      <c r="F38" s="605"/>
-      <c r="G38" s="606"/>
+      <c r="D38" s="606"/>
+      <c r="E38" s="606"/>
+      <c r="F38" s="606"/>
+      <c r="G38" s="607"/>
       <c r="H38" s="506" t="s">
         <v>184</v>
       </c>
@@ -10083,13 +10093,13 @@
       <c r="B39" s="505">
         <v>9</v>
       </c>
-      <c r="C39" s="604" t="s">
+      <c r="C39" s="605" t="s">
         <v>267</v>
       </c>
-      <c r="D39" s="605"/>
-      <c r="E39" s="605"/>
-      <c r="F39" s="605"/>
-      <c r="G39" s="606"/>
+      <c r="D39" s="606"/>
+      <c r="E39" s="606"/>
+      <c r="F39" s="606"/>
+      <c r="G39" s="607"/>
       <c r="H39" s="506" t="s">
         <v>56</v>
       </c>
@@ -10119,31 +10129,31 @@
     </row>
     <row r="41" spans="1:23" ht="17.25" customHeight="1">
       <c r="A41" s="504"/>
-      <c r="B41" s="603" t="s">
+      <c r="B41" s="615" t="s">
         <v>268</v>
       </c>
-      <c r="C41" s="603"/>
-      <c r="D41" s="603"/>
-      <c r="E41" s="603"/>
-      <c r="F41" s="603"/>
+      <c r="C41" s="615"/>
+      <c r="D41" s="615"/>
+      <c r="E41" s="615"/>
+      <c r="F41" s="615"/>
       <c r="G41" s="515"/>
-      <c r="H41" s="607" t="s">
+      <c r="H41" s="616" t="s">
         <v>269</v>
       </c>
-      <c r="I41" s="608"/>
-      <c r="J41" s="609"/>
-      <c r="K41" s="609"/>
-      <c r="L41" s="608"/>
+      <c r="I41" s="617"/>
+      <c r="J41" s="618"/>
+      <c r="K41" s="618"/>
+      <c r="L41" s="617"/>
       <c r="M41" s="87"/>
       <c r="W41" s="435"/>
     </row>
     <row r="42" spans="1:23" ht="26.25" customHeight="1">
       <c r="A42" s="504"/>
-      <c r="B42" s="610" t="s">
+      <c r="B42" s="619" t="s">
         <v>270</v>
       </c>
-      <c r="C42" s="610"/>
-      <c r="D42" s="610"/>
+      <c r="C42" s="619"/>
+      <c r="D42" s="619"/>
       <c r="E42" s="516" t="s">
         <v>271</v>
       </c>
@@ -10151,23 +10161,23 @@
         <v>272</v>
       </c>
       <c r="G42" s="515"/>
-      <c r="H42" s="598" t="s">
+      <c r="H42" s="610" t="s">
         <v>273</v>
       </c>
-      <c r="I42" s="598"/>
-      <c r="J42" s="611"/>
-      <c r="K42" s="611"/>
-      <c r="L42" s="611"/>
+      <c r="I42" s="610"/>
+      <c r="J42" s="620"/>
+      <c r="K42" s="620"/>
+      <c r="L42" s="620"/>
       <c r="M42" s="87"/>
       <c r="W42" s="435"/>
     </row>
     <row r="43" spans="1:23" ht="15" customHeight="1">
       <c r="A43" s="504"/>
-      <c r="B43" s="596" t="s">
+      <c r="B43" s="626" t="s">
         <v>274</v>
       </c>
-      <c r="C43" s="596"/>
-      <c r="D43" s="596"/>
+      <c r="C43" s="626"/>
+      <c r="D43" s="626"/>
       <c r="E43" s="517" t="s">
         <v>142</v>
       </c>
@@ -10175,23 +10185,23 @@
         <v>275</v>
       </c>
       <c r="G43" s="515"/>
-      <c r="H43" s="598" t="s">
+      <c r="H43" s="610" t="s">
         <v>276</v>
       </c>
-      <c r="I43" s="598"/>
-      <c r="J43" s="599"/>
-      <c r="K43" s="599"/>
-      <c r="L43" s="600"/>
+      <c r="I43" s="610"/>
+      <c r="J43" s="611"/>
+      <c r="K43" s="611"/>
+      <c r="L43" s="612"/>
       <c r="M43" s="87"/>
       <c r="W43" s="435"/>
     </row>
     <row r="44" spans="1:23" ht="15" customHeight="1">
       <c r="A44" s="504"/>
-      <c r="B44" s="596" t="s">
+      <c r="B44" s="626" t="s">
         <v>277</v>
       </c>
-      <c r="C44" s="596"/>
-      <c r="D44" s="596"/>
+      <c r="C44" s="626"/>
+      <c r="D44" s="626"/>
       <c r="E44" s="517" t="s">
         <v>144</v>
       </c>
@@ -10199,20 +10209,20 @@
         <v>275</v>
       </c>
       <c r="G44" s="515"/>
-      <c r="H44" s="598"/>
-      <c r="I44" s="598"/>
-      <c r="J44" s="601"/>
-      <c r="K44" s="601"/>
-      <c r="L44" s="602"/>
+      <c r="H44" s="610"/>
+      <c r="I44" s="610"/>
+      <c r="J44" s="613"/>
+      <c r="K44" s="613"/>
+      <c r="L44" s="614"/>
       <c r="M44" s="87"/>
     </row>
     <row r="45" spans="1:23" ht="15" customHeight="1">
       <c r="A45" s="504"/>
-      <c r="B45" s="592" t="s">
+      <c r="B45" s="622" t="s">
         <v>278</v>
       </c>
-      <c r="C45" s="592"/>
-      <c r="D45" s="592"/>
+      <c r="C45" s="622"/>
+      <c r="D45" s="622"/>
       <c r="E45" s="517" t="s">
         <v>146</v>
       </c>
@@ -10220,39 +10230,39 @@
         <v>275</v>
       </c>
       <c r="G45" s="515"/>
-      <c r="H45" s="598" t="s">
+      <c r="H45" s="610" t="s">
         <v>279</v>
       </c>
-      <c r="I45" s="598"/>
-      <c r="J45" s="599"/>
-      <c r="K45" s="599"/>
-      <c r="L45" s="600"/>
+      <c r="I45" s="610"/>
+      <c r="J45" s="611"/>
+      <c r="K45" s="611"/>
+      <c r="L45" s="612"/>
       <c r="M45" s="87"/>
     </row>
     <row r="46" spans="1:23" ht="15" customHeight="1">
       <c r="A46" s="504"/>
-      <c r="B46" s="603" t="s">
+      <c r="B46" s="615" t="s">
         <v>280</v>
       </c>
-      <c r="C46" s="603"/>
-      <c r="D46" s="603"/>
-      <c r="E46" s="603"/>
-      <c r="F46" s="603"/>
+      <c r="C46" s="615"/>
+      <c r="D46" s="615"/>
+      <c r="E46" s="615"/>
+      <c r="F46" s="615"/>
       <c r="G46" s="515"/>
-      <c r="H46" s="598"/>
-      <c r="I46" s="598"/>
-      <c r="J46" s="601"/>
-      <c r="K46" s="601"/>
-      <c r="L46" s="602"/>
+      <c r="H46" s="610"/>
+      <c r="I46" s="610"/>
+      <c r="J46" s="613"/>
+      <c r="K46" s="613"/>
+      <c r="L46" s="614"/>
       <c r="M46" s="87"/>
     </row>
     <row r="47" spans="1:23" ht="15" customHeight="1">
       <c r="A47" s="504"/>
-      <c r="B47" s="592" t="s">
+      <c r="B47" s="622" t="s">
         <v>281</v>
       </c>
-      <c r="C47" s="592"/>
-      <c r="D47" s="592"/>
+      <c r="C47" s="622"/>
+      <c r="D47" s="622"/>
       <c r="E47" s="517" t="s">
         <v>148</v>
       </c>
@@ -10260,20 +10270,20 @@
         <v>282</v>
       </c>
       <c r="G47" s="515"/>
-      <c r="H47" s="593"/>
-      <c r="I47" s="593"/>
-      <c r="J47" s="594"/>
-      <c r="K47" s="594"/>
-      <c r="L47" s="595"/>
+      <c r="H47" s="623"/>
+      <c r="I47" s="623"/>
+      <c r="J47" s="624"/>
+      <c r="K47" s="624"/>
+      <c r="L47" s="625"/>
       <c r="M47" s="87"/>
     </row>
     <row r="48" spans="1:23" ht="15" customHeight="1">
       <c r="A48" s="504"/>
-      <c r="B48" s="596" t="s">
+      <c r="B48" s="626" t="s">
         <v>149</v>
       </c>
-      <c r="C48" s="596"/>
-      <c r="D48" s="596"/>
+      <c r="C48" s="626"/>
+      <c r="D48" s="626"/>
       <c r="E48" s="517" t="s">
         <v>146</v>
       </c>
@@ -10281,20 +10291,20 @@
         <v>282</v>
       </c>
       <c r="G48" s="515"/>
-      <c r="H48" s="593"/>
-      <c r="I48" s="593"/>
-      <c r="J48" s="594"/>
-      <c r="K48" s="594"/>
-      <c r="L48" s="595"/>
+      <c r="H48" s="623"/>
+      <c r="I48" s="623"/>
+      <c r="J48" s="624"/>
+      <c r="K48" s="624"/>
+      <c r="L48" s="625"/>
       <c r="M48" s="87"/>
     </row>
     <row r="49" spans="1:13" ht="15" customHeight="1">
       <c r="A49" s="504"/>
-      <c r="B49" s="596" t="s">
+      <c r="B49" s="626" t="s">
         <v>151</v>
       </c>
-      <c r="C49" s="596"/>
-      <c r="D49" s="596"/>
+      <c r="C49" s="626"/>
+      <c r="D49" s="626"/>
       <c r="E49" s="517" t="s">
         <v>146</v>
       </c>
@@ -10412,15 +10422,15 @@
       <c r="M56" s="87"/>
     </row>
     <row r="57" spans="1:13" ht="4.5" customHeight="1">
-      <c r="B57" s="597"/>
-      <c r="C57" s="597"/>
-      <c r="D57" s="597"/>
-      <c r="E57" s="597"/>
-      <c r="F57" s="597"/>
-      <c r="G57" s="597"/>
-      <c r="H57" s="597"/>
-      <c r="I57" s="597"/>
-      <c r="J57" s="597"/>
+      <c r="B57" s="627"/>
+      <c r="C57" s="627"/>
+      <c r="D57" s="627"/>
+      <c r="E57" s="627"/>
+      <c r="F57" s="627"/>
+      <c r="G57" s="627"/>
+      <c r="H57" s="627"/>
+      <c r="I57" s="627"/>
+      <c r="J57" s="627"/>
       <c r="K57" s="480"/>
       <c r="L57" s="435"/>
       <c r="M57" s="87"/>
@@ -10463,20 +10473,20 @@
     </row>
     <row r="60" spans="1:13" ht="3.75" customHeight="1"/>
     <row r="61" spans="1:13" ht="30.75" customHeight="1">
-      <c r="A61" s="589" t="s">
+      <c r="A61" s="621" t="s">
         <v>285</v>
       </c>
-      <c r="B61" s="589"/>
-      <c r="C61" s="589"/>
-      <c r="D61" s="589"/>
-      <c r="E61" s="589"/>
-      <c r="F61" s="589"/>
-      <c r="G61" s="589"/>
-      <c r="H61" s="589"/>
-      <c r="I61" s="589"/>
-      <c r="J61" s="589"/>
-      <c r="K61" s="589"/>
-      <c r="L61" s="589"/>
+      <c r="B61" s="621"/>
+      <c r="C61" s="621"/>
+      <c r="D61" s="621"/>
+      <c r="E61" s="621"/>
+      <c r="F61" s="621"/>
+      <c r="G61" s="621"/>
+      <c r="H61" s="621"/>
+      <c r="I61" s="621"/>
+      <c r="J61" s="621"/>
+      <c r="K61" s="621"/>
+      <c r="L61" s="621"/>
     </row>
     <row r="62" spans="1:13" ht="15.9" customHeight="1"/>
     <row r="63" spans="1:13" ht="15.9" customHeight="1"/>
@@ -10486,40 +10496,6 @@
     <protectedRange sqref="C57" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="50">
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A7:L7"/>
-    <mergeCell ref="A8:L8"/>
-    <mergeCell ref="A14:L14"/>
-    <mergeCell ref="A15:L15"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="H25:J25"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="C37:G37"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="B30:G30"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="C32:G32"/>
-    <mergeCell ref="C33:G33"/>
-    <mergeCell ref="C34:G34"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="H45:I46"/>
-    <mergeCell ref="J45:L46"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="C38:G38"/>
-    <mergeCell ref="C39:G39"/>
-    <mergeCell ref="B41:F41"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="J41:L41"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="J42:L42"/>
     <mergeCell ref="A61:L61"/>
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="E28:F28"/>
@@ -10536,6 +10512,40 @@
     <mergeCell ref="J43:L44"/>
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="B45:D45"/>
+    <mergeCell ref="H45:I46"/>
+    <mergeCell ref="J45:L46"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="C38:G38"/>
+    <mergeCell ref="C39:G39"/>
+    <mergeCell ref="B41:F41"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="J41:L41"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="J42:L42"/>
+    <mergeCell ref="C37:G37"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="C31:G31"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="C33:G33"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="H25:J25"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A8:L8"/>
+    <mergeCell ref="A14:L14"/>
+    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A17:I17"/>
   </mergeCells>
   <conditionalFormatting sqref="A18:A22">
     <cfRule type="cellIs" priority="1" stopIfTrue="1" operator="between">
@@ -10589,40 +10599,40 @@
       <c r="N1" s="309"/>
     </row>
     <row r="2" spans="1:17" ht="15.9" customHeight="1">
-      <c r="A2" s="567" t="s">
+      <c r="A2" s="544" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="567"/>
-      <c r="C2" s="567"/>
-      <c r="D2" s="567"/>
-      <c r="E2" s="567"/>
-      <c r="F2" s="567"/>
-      <c r="G2" s="567"/>
-      <c r="H2" s="567"/>
-      <c r="I2" s="567"/>
-      <c r="J2" s="567"/>
-      <c r="K2" s="567"/>
-      <c r="L2" s="567"/>
-      <c r="M2" s="567"/>
-      <c r="N2" s="567"/>
+      <c r="B2" s="544"/>
+      <c r="C2" s="544"/>
+      <c r="D2" s="544"/>
+      <c r="E2" s="544"/>
+      <c r="F2" s="544"/>
+      <c r="G2" s="544"/>
+      <c r="H2" s="544"/>
+      <c r="I2" s="544"/>
+      <c r="J2" s="544"/>
+      <c r="K2" s="544"/>
+      <c r="L2" s="544"/>
+      <c r="M2" s="544"/>
+      <c r="N2" s="544"/>
     </row>
     <row r="3" spans="1:17" ht="15.9" customHeight="1">
-      <c r="A3" s="631">
+      <c r="A3" s="637">
         <v>0</v>
       </c>
-      <c r="B3" s="631"/>
-      <c r="C3" s="631"/>
-      <c r="D3" s="631"/>
-      <c r="E3" s="631"/>
-      <c r="F3" s="631"/>
-      <c r="G3" s="631"/>
-      <c r="H3" s="631"/>
-      <c r="I3" s="631"/>
-      <c r="J3" s="631"/>
-      <c r="K3" s="631"/>
-      <c r="L3" s="631"/>
-      <c r="M3" s="631"/>
-      <c r="N3" s="631"/>
+      <c r="B3" s="637"/>
+      <c r="C3" s="637"/>
+      <c r="D3" s="637"/>
+      <c r="E3" s="637"/>
+      <c r="F3" s="637"/>
+      <c r="G3" s="637"/>
+      <c r="H3" s="637"/>
+      <c r="I3" s="637"/>
+      <c r="J3" s="637"/>
+      <c r="K3" s="637"/>
+      <c r="L3" s="637"/>
+      <c r="M3" s="637"/>
+      <c r="N3" s="637"/>
     </row>
     <row r="4" spans="1:17" ht="15.9" customHeight="1"/>
     <row r="5" spans="1:17" ht="15" customHeight="1">
@@ -10632,18 +10642,18 @@
       <c r="B5" s="177" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="706">
+      <c r="C5" s="628">
         <f>+Resumen!P2</f>
         <v>0</v>
       </c>
-      <c r="D5" s="706"/>
-      <c r="E5" s="706"/>
-      <c r="F5" s="706"/>
-      <c r="G5" s="706"/>
-      <c r="H5" s="706"/>
-      <c r="I5" s="706"/>
-      <c r="J5" s="706"/>
-      <c r="K5" s="706"/>
+      <c r="D5" s="628"/>
+      <c r="E5" s="628"/>
+      <c r="F5" s="628"/>
+      <c r="G5" s="628"/>
+      <c r="H5" s="628"/>
+      <c r="I5" s="628"/>
+      <c r="J5" s="628"/>
+      <c r="K5" s="628"/>
       <c r="L5" s="27" t="s">
         <v>6</v>
       </c>
@@ -10662,18 +10672,18 @@
       <c r="B6" s="177" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="628">
+      <c r="C6" s="630">
         <f>+Resumen!P3</f>
         <v>0</v>
       </c>
-      <c r="D6" s="628"/>
-      <c r="E6" s="628"/>
-      <c r="F6" s="628"/>
-      <c r="G6" s="628"/>
-      <c r="H6" s="628"/>
-      <c r="I6" s="628"/>
-      <c r="J6" s="628"/>
-      <c r="K6" s="628"/>
+      <c r="D6" s="630"/>
+      <c r="E6" s="630"/>
+      <c r="F6" s="630"/>
+      <c r="G6" s="630"/>
+      <c r="H6" s="630"/>
+      <c r="I6" s="630"/>
+      <c r="J6" s="630"/>
+      <c r="K6" s="630"/>
       <c r="L6" s="458" t="s">
         <v>233</v>
       </c>
@@ -10695,18 +10705,18 @@
       <c r="B7" s="177" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="706">
+      <c r="C7" s="628">
         <f>+Resumen!P4</f>
         <v>0</v>
       </c>
-      <c r="D7" s="706"/>
-      <c r="E7" s="706"/>
-      <c r="F7" s="706"/>
-      <c r="G7" s="706"/>
-      <c r="H7" s="706"/>
-      <c r="I7" s="706"/>
-      <c r="J7" s="706"/>
-      <c r="K7" s="706"/>
+      <c r="D7" s="628"/>
+      <c r="E7" s="628"/>
+      <c r="F7" s="628"/>
+      <c r="G7" s="628"/>
+      <c r="H7" s="628"/>
+      <c r="I7" s="628"/>
+      <c r="J7" s="628"/>
+      <c r="K7" s="628"/>
       <c r="L7" s="458" t="s">
         <v>297</v>
       </c>
@@ -10728,18 +10738,18 @@
       <c r="B8" s="177" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="628">
+      <c r="C8" s="630">
         <f>+Resumen!P5</f>
         <v>0</v>
       </c>
-      <c r="D8" s="628"/>
-      <c r="E8" s="628"/>
-      <c r="F8" s="628"/>
-      <c r="G8" s="628"/>
-      <c r="H8" s="628"/>
-      <c r="I8" s="628"/>
-      <c r="J8" s="628"/>
-      <c r="K8" s="628"/>
+      <c r="D8" s="630"/>
+      <c r="E8" s="630"/>
+      <c r="F8" s="630"/>
+      <c r="G8" s="630"/>
+      <c r="H8" s="630"/>
+      <c r="I8" s="630"/>
+      <c r="J8" s="630"/>
+      <c r="K8" s="630"/>
       <c r="L8" s="458" t="s">
         <v>101</v>
       </c>
@@ -10776,43 +10786,43 @@
       <c r="Q9" s="317"/>
     </row>
     <row r="10" spans="1:17">
-      <c r="A10" s="632" t="s">
+      <c r="A10" s="638" t="s">
         <v>102</v>
       </c>
-      <c r="B10" s="633"/>
-      <c r="C10" s="633"/>
-      <c r="D10" s="633"/>
-      <c r="E10" s="633"/>
-      <c r="F10" s="633"/>
-      <c r="G10" s="633"/>
-      <c r="H10" s="633"/>
-      <c r="I10" s="633"/>
-      <c r="J10" s="633"/>
-      <c r="K10" s="633"/>
-      <c r="L10" s="633"/>
-      <c r="M10" s="633"/>
-      <c r="N10" s="634"/>
+      <c r="B10" s="639"/>
+      <c r="C10" s="639"/>
+      <c r="D10" s="639"/>
+      <c r="E10" s="639"/>
+      <c r="F10" s="639"/>
+      <c r="G10" s="639"/>
+      <c r="H10" s="639"/>
+      <c r="I10" s="639"/>
+      <c r="J10" s="639"/>
+      <c r="K10" s="639"/>
+      <c r="L10" s="639"/>
+      <c r="M10" s="639"/>
+      <c r="N10" s="640"/>
       <c r="O10" s="317"/>
       <c r="P10" s="317"/>
       <c r="Q10" s="317"/>
     </row>
     <row r="11" spans="1:17" ht="12" customHeight="1">
-      <c r="A11" s="635" t="s">
+      <c r="A11" s="641" t="s">
         <v>103</v>
       </c>
-      <c r="B11" s="636"/>
-      <c r="C11" s="636"/>
-      <c r="D11" s="636"/>
-      <c r="E11" s="636"/>
-      <c r="F11" s="636"/>
-      <c r="G11" s="636"/>
-      <c r="H11" s="636"/>
-      <c r="I11" s="636"/>
-      <c r="J11" s="636"/>
-      <c r="K11" s="636"/>
-      <c r="L11" s="636"/>
-      <c r="M11" s="636"/>
-      <c r="N11" s="637"/>
+      <c r="B11" s="642"/>
+      <c r="C11" s="642"/>
+      <c r="D11" s="642"/>
+      <c r="E11" s="642"/>
+      <c r="F11" s="642"/>
+      <c r="G11" s="642"/>
+      <c r="H11" s="642"/>
+      <c r="I11" s="642"/>
+      <c r="J11" s="642"/>
+      <c r="K11" s="642"/>
+      <c r="L11" s="642"/>
+      <c r="M11" s="642"/>
+      <c r="N11" s="643"/>
       <c r="O11" s="317"/>
       <c r="P11" s="317"/>
       <c r="Q11" s="317"/>
@@ -10982,16 +10992,16 @@
       <c r="A18" s="310"/>
       <c r="B18" s="310"/>
       <c r="C18" s="310"/>
-      <c r="D18" s="641"/>
-      <c r="E18" s="641"/>
+      <c r="D18" s="646"/>
+      <c r="E18" s="646"/>
       <c r="F18" s="310"/>
       <c r="G18" s="310"/>
       <c r="H18" s="310"/>
       <c r="I18" s="310"/>
       <c r="J18" s="310"/>
       <c r="K18" s="310"/>
-      <c r="L18" s="641"/>
-      <c r="M18" s="641"/>
+      <c r="L18" s="646"/>
+      <c r="M18" s="646"/>
       <c r="N18" s="310"/>
       <c r="O18" s="317"/>
       <c r="P18" s="317"/>
@@ -11001,14 +11011,14 @@
       <c r="A19" s="310"/>
       <c r="B19" s="310"/>
       <c r="C19" s="310"/>
-      <c r="D19" s="642" t="s">
+      <c r="D19" s="647" t="s">
         <v>108</v>
       </c>
-      <c r="E19" s="642"/>
-      <c r="F19" s="642"/>
-      <c r="G19" s="642"/>
-      <c r="H19" s="642"/>
-      <c r="I19" s="642"/>
+      <c r="E19" s="647"/>
+      <c r="F19" s="647"/>
+      <c r="G19" s="647"/>
+      <c r="H19" s="647"/>
+      <c r="I19" s="647"/>
       <c r="J19" s="311" t="s">
         <v>109</v>
       </c>
@@ -11041,8 +11051,8 @@
         <f>+'Datos ensayo'!G17</f>
         <v>1</v>
       </c>
-      <c r="L20" s="639"/>
-      <c r="M20" s="639"/>
+      <c r="L20" s="644"/>
+      <c r="M20" s="644"/>
       <c r="N20" s="312"/>
       <c r="O20" s="317"/>
       <c r="P20" s="317"/>
@@ -11067,8 +11077,8 @@
         <f>+'Datos ensayo'!G18</f>
         <v>0</v>
       </c>
-      <c r="L21" s="639"/>
-      <c r="M21" s="639"/>
+      <c r="L21" s="644"/>
+      <c r="M21" s="644"/>
       <c r="N21" s="312"/>
       <c r="O21" s="317"/>
       <c r="P21" s="317"/>
@@ -11093,8 +11103,8 @@
         <f>+'Datos ensayo'!H19</f>
         <v>0,00</v>
       </c>
-      <c r="L22" s="640"/>
-      <c r="M22" s="640"/>
+      <c r="L22" s="645"/>
+      <c r="M22" s="645"/>
       <c r="N22" s="313"/>
       <c r="O22" s="323"/>
       <c r="P22" s="323"/>
@@ -11443,11 +11453,11 @@
       <c r="H37" s="193"/>
       <c r="I37" s="195"/>
       <c r="J37" s="195"/>
-      <c r="K37" s="644">
+      <c r="K37" s="629">
         <f>+Resumen!E27</f>
         <v>0</v>
       </c>
-      <c r="L37" s="644"/>
+      <c r="L37" s="629"/>
       <c r="M37" s="159"/>
       <c r="N37" s="159"/>
       <c r="O37" s="317"/>
@@ -11467,11 +11477,11 @@
       <c r="H38" s="193"/>
       <c r="I38" s="195"/>
       <c r="J38" s="195"/>
-      <c r="K38" s="643">
+      <c r="K38" s="648">
         <f>+Resumen!E28</f>
         <v>0</v>
       </c>
-      <c r="L38" s="643"/>
+      <c r="L38" s="648"/>
       <c r="M38" s="159"/>
       <c r="N38" s="159"/>
       <c r="O38" s="317"/>
@@ -11507,106 +11517,106 @@
       <c r="Q40" s="317"/>
     </row>
     <row r="41" spans="1:17" ht="15" customHeight="1">
-      <c r="A41" s="629" t="s">
+      <c r="A41" s="636" t="s">
         <v>312</v>
       </c>
-      <c r="B41" s="629"/>
-      <c r="C41" s="629"/>
-      <c r="D41" s="629"/>
-      <c r="E41" s="629"/>
-      <c r="F41" s="629"/>
-      <c r="G41" s="629"/>
-      <c r="H41" s="629"/>
-      <c r="I41" s="629"/>
-      <c r="J41" s="629"/>
-      <c r="K41" s="629"/>
-      <c r="L41" s="629"/>
-      <c r="M41" s="629"/>
-      <c r="N41" s="629"/>
+      <c r="B41" s="636"/>
+      <c r="C41" s="636"/>
+      <c r="D41" s="636"/>
+      <c r="E41" s="636"/>
+      <c r="F41" s="636"/>
+      <c r="G41" s="636"/>
+      <c r="H41" s="636"/>
+      <c r="I41" s="636"/>
+      <c r="J41" s="636"/>
+      <c r="K41" s="636"/>
+      <c r="L41" s="636"/>
+      <c r="M41" s="636"/>
+      <c r="N41" s="636"/>
       <c r="O41" s="317"/>
       <c r="P41" s="317"/>
       <c r="Q41" s="317"/>
     </row>
     <row r="42" spans="1:17" ht="33" customHeight="1">
-      <c r="A42" s="638" t="s">
+      <c r="A42" s="633" t="s">
         <v>313</v>
       </c>
-      <c r="B42" s="638"/>
-      <c r="C42" s="638"/>
-      <c r="D42" s="638"/>
-      <c r="E42" s="638"/>
-      <c r="F42" s="638"/>
-      <c r="G42" s="638"/>
-      <c r="H42" s="638"/>
-      <c r="I42" s="638"/>
-      <c r="J42" s="638"/>
-      <c r="K42" s="638"/>
-      <c r="L42" s="638"/>
-      <c r="M42" s="638"/>
-      <c r="N42" s="638"/>
+      <c r="B42" s="633"/>
+      <c r="C42" s="633"/>
+      <c r="D42" s="633"/>
+      <c r="E42" s="633"/>
+      <c r="F42" s="633"/>
+      <c r="G42" s="633"/>
+      <c r="H42" s="633"/>
+      <c r="I42" s="633"/>
+      <c r="J42" s="633"/>
+      <c r="K42" s="633"/>
+      <c r="L42" s="633"/>
+      <c r="M42" s="633"/>
+      <c r="N42" s="633"/>
       <c r="O42" s="317"/>
       <c r="P42" s="317"/>
       <c r="Q42" s="317"/>
     </row>
     <row r="43" spans="1:17" ht="18.600000000000001" customHeight="1">
-      <c r="A43" s="638" t="s">
+      <c r="A43" s="633" t="s">
         <v>314</v>
       </c>
-      <c r="B43" s="638"/>
-      <c r="C43" s="638"/>
-      <c r="D43" s="638"/>
-      <c r="E43" s="638"/>
-      <c r="F43" s="638"/>
-      <c r="G43" s="638"/>
-      <c r="H43" s="638"/>
-      <c r="I43" s="638"/>
-      <c r="J43" s="638"/>
-      <c r="K43" s="638"/>
-      <c r="L43" s="638"/>
-      <c r="M43" s="638"/>
-      <c r="N43" s="638"/>
+      <c r="B43" s="633"/>
+      <c r="C43" s="633"/>
+      <c r="D43" s="633"/>
+      <c r="E43" s="633"/>
+      <c r="F43" s="633"/>
+      <c r="G43" s="633"/>
+      <c r="H43" s="633"/>
+      <c r="I43" s="633"/>
+      <c r="J43" s="633"/>
+      <c r="K43" s="633"/>
+      <c r="L43" s="633"/>
+      <c r="M43" s="633"/>
+      <c r="N43" s="633"/>
       <c r="O43" s="317"/>
       <c r="P43" s="317"/>
       <c r="Q43" s="317"/>
     </row>
     <row r="44" spans="1:17" ht="23.4" customHeight="1">
-      <c r="A44" s="638" t="s">
+      <c r="A44" s="633" t="s">
         <v>315</v>
       </c>
-      <c r="B44" s="638"/>
-      <c r="C44" s="638"/>
-      <c r="D44" s="638"/>
-      <c r="E44" s="638"/>
-      <c r="F44" s="638"/>
-      <c r="G44" s="638"/>
-      <c r="H44" s="638"/>
-      <c r="I44" s="638"/>
-      <c r="J44" s="638"/>
-      <c r="K44" s="638"/>
-      <c r="L44" s="638"/>
-      <c r="M44" s="638"/>
-      <c r="N44" s="638"/>
+      <c r="B44" s="633"/>
+      <c r="C44" s="633"/>
+      <c r="D44" s="633"/>
+      <c r="E44" s="633"/>
+      <c r="F44" s="633"/>
+      <c r="G44" s="633"/>
+      <c r="H44" s="633"/>
+      <c r="I44" s="633"/>
+      <c r="J44" s="633"/>
+      <c r="K44" s="633"/>
+      <c r="L44" s="633"/>
+      <c r="M44" s="633"/>
+      <c r="N44" s="633"/>
       <c r="O44" s="317"/>
       <c r="P44" s="317"/>
       <c r="Q44" s="317"/>
     </row>
     <row r="45" spans="1:17" ht="23.25" customHeight="1">
-      <c r="A45" s="647" t="s">
+      <c r="A45" s="635" t="s">
         <v>316</v>
       </c>
-      <c r="B45" s="647"/>
-      <c r="C45" s="647"/>
-      <c r="D45" s="647"/>
-      <c r="E45" s="647"/>
-      <c r="F45" s="647"/>
-      <c r="G45" s="647"/>
-      <c r="H45" s="647"/>
-      <c r="I45" s="647"/>
-      <c r="J45" s="647"/>
-      <c r="K45" s="647"/>
-      <c r="L45" s="647"/>
-      <c r="M45" s="647"/>
-      <c r="N45" s="647"/>
+      <c r="B45" s="635"/>
+      <c r="C45" s="635"/>
+      <c r="D45" s="635"/>
+      <c r="E45" s="635"/>
+      <c r="F45" s="635"/>
+      <c r="G45" s="635"/>
+      <c r="H45" s="635"/>
+      <c r="I45" s="635"/>
+      <c r="J45" s="635"/>
+      <c r="K45" s="635"/>
+      <c r="L45" s="635"/>
+      <c r="M45" s="635"/>
+      <c r="N45" s="635"/>
       <c r="O45" s="317"/>
       <c r="P45" s="317"/>
       <c r="Q45" s="317"/>
@@ -11644,10 +11654,10 @@
       <c r="A48" s="196"/>
       <c r="B48" s="196"/>
       <c r="C48" s="196"/>
-      <c r="K48" s="630"/>
-      <c r="L48" s="630"/>
-      <c r="M48" s="630"/>
-      <c r="N48" s="630"/>
+      <c r="K48" s="634"/>
+      <c r="L48" s="634"/>
+      <c r="M48" s="634"/>
+      <c r="N48" s="634"/>
       <c r="O48" s="317"/>
       <c r="P48" s="317"/>
       <c r="Q48" s="317"/>
@@ -11669,10 +11679,10 @@
       <c r="A50" s="196"/>
       <c r="B50" s="196"/>
       <c r="C50" s="196"/>
-      <c r="K50" s="630"/>
-      <c r="L50" s="630"/>
-      <c r="M50" s="630"/>
-      <c r="N50" s="630"/>
+      <c r="K50" s="634"/>
+      <c r="L50" s="634"/>
+      <c r="M50" s="634"/>
+      <c r="N50" s="634"/>
       <c r="O50" s="317"/>
       <c r="P50" s="317"/>
       <c r="Q50" s="317"/>
@@ -11690,10 +11700,10 @@
       <c r="H51" s="324"/>
       <c r="I51" s="324"/>
       <c r="J51" s="324"/>
-      <c r="K51" s="630"/>
-      <c r="L51" s="630"/>
-      <c r="M51" s="630"/>
-      <c r="N51" s="630"/>
+      <c r="K51" s="634"/>
+      <c r="L51" s="634"/>
+      <c r="M51" s="634"/>
+      <c r="N51" s="634"/>
     </row>
     <row r="52" spans="1:17" ht="11.25" customHeight="1">
       <c r="A52" s="195" t="s">
@@ -11708,18 +11718,19 @@
       <c r="H52" s="324"/>
       <c r="I52" s="324"/>
       <c r="J52" s="324"/>
-      <c r="K52" s="630" t="s">
+      <c r="K52" s="634" t="s">
         <v>125</v>
       </c>
-      <c r="L52" s="630"/>
-      <c r="M52" s="630"/>
-      <c r="N52" s="630"/>
+      <c r="L52" s="634"/>
+      <c r="M52" s="634"/>
+      <c r="N52" s="634"/>
     </row>
     <row r="53" spans="1:17" ht="15.9" customHeight="1">
       <c r="M53" s="185"/>
       <c r="N53" s="317"/>
     </row>
     <row r="54" spans="1:17">
+      <c r="H54" s="707"/>
       <c r="M54" s="186"/>
       <c r="N54" s="317"/>
     </row>
@@ -11763,20 +11774,20 @@
       <c r="N58" s="187"/>
     </row>
     <row r="59" spans="1:17" ht="30" customHeight="1">
-      <c r="A59" s="646"/>
-      <c r="B59" s="646"/>
-      <c r="C59" s="646"/>
-      <c r="D59" s="646"/>
-      <c r="E59" s="646"/>
-      <c r="F59" s="646"/>
-      <c r="G59" s="646"/>
-      <c r="H59" s="646"/>
-      <c r="I59" s="646"/>
-      <c r="J59" s="646"/>
-      <c r="K59" s="646"/>
-      <c r="L59" s="646"/>
-      <c r="M59" s="646"/>
-      <c r="N59" s="646"/>
+      <c r="A59" s="632"/>
+      <c r="B59" s="632"/>
+      <c r="C59" s="632"/>
+      <c r="D59" s="632"/>
+      <c r="E59" s="632"/>
+      <c r="F59" s="632"/>
+      <c r="G59" s="632"/>
+      <c r="H59" s="632"/>
+      <c r="I59" s="632"/>
+      <c r="J59" s="632"/>
+      <c r="K59" s="632"/>
+      <c r="L59" s="632"/>
+      <c r="M59" s="632"/>
+      <c r="N59" s="632"/>
     </row>
     <row r="60" spans="1:17" ht="30" customHeight="1">
       <c r="A60" s="193"/>
@@ -11795,20 +11806,20 @@
       <c r="N60" s="324"/>
     </row>
     <row r="61" spans="1:17" ht="39.75" customHeight="1">
-      <c r="A61" s="646"/>
-      <c r="B61" s="646"/>
-      <c r="C61" s="646"/>
-      <c r="D61" s="646"/>
-      <c r="E61" s="646"/>
-      <c r="F61" s="646"/>
-      <c r="G61" s="646"/>
-      <c r="H61" s="646"/>
-      <c r="I61" s="646"/>
-      <c r="J61" s="646"/>
-      <c r="K61" s="646"/>
-      <c r="L61" s="646"/>
-      <c r="M61" s="646"/>
-      <c r="N61" s="646"/>
+      <c r="A61" s="632"/>
+      <c r="B61" s="632"/>
+      <c r="C61" s="632"/>
+      <c r="D61" s="632"/>
+      <c r="E61" s="632"/>
+      <c r="F61" s="632"/>
+      <c r="G61" s="632"/>
+      <c r="H61" s="632"/>
+      <c r="I61" s="632"/>
+      <c r="J61" s="632"/>
+      <c r="K61" s="632"/>
+      <c r="L61" s="632"/>
+      <c r="M61" s="632"/>
+      <c r="N61" s="632"/>
     </row>
     <row r="62" spans="1:17" ht="30" customHeight="1">
       <c r="A62" s="194"/>
@@ -11897,15 +11908,15 @@
       <c r="N78" s="317"/>
     </row>
     <row r="79" spans="11:14">
-      <c r="K79" s="645"/>
-      <c r="L79" s="645"/>
-      <c r="M79" s="645"/>
+      <c r="K79" s="631"/>
+      <c r="L79" s="631"/>
+      <c r="M79" s="631"/>
       <c r="N79" s="317"/>
     </row>
     <row r="80" spans="11:14">
-      <c r="K80" s="645"/>
-      <c r="L80" s="645"/>
-      <c r="M80" s="645"/>
+      <c r="K80" s="631"/>
+      <c r="L80" s="631"/>
+      <c r="M80" s="631"/>
       <c r="N80" s="317"/>
     </row>
     <row r="81" spans="1:14">
@@ -12023,30 +12034,11 @@
       <c r="N94" s="317"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="t8jSAIyVyB5oMAyJpHM2Ug4y00Rel+1Ax2C/5TZDOGsIV0U2WwRM4IKzDsynSPYlwDGtgRkiUamwVw2TCWPvtg==" saltValue="pVIlk7q0zbEYwQVNo0WkrA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <protectedRanges>
     <protectedRange sqref="E7:F9 E12:F12" name="Rango3_3_1_1_1_1_1_1_1_1"/>
     <protectedRange sqref="E5:F6" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="30">
-    <mergeCell ref="C5:K5"/>
-    <mergeCell ref="K37:L37"/>
-    <mergeCell ref="C6:K6"/>
-    <mergeCell ref="K79:K80"/>
-    <mergeCell ref="L79:L80"/>
-    <mergeCell ref="M79:M80"/>
-    <mergeCell ref="A59:N59"/>
-    <mergeCell ref="A61:N61"/>
-    <mergeCell ref="A42:N42"/>
-    <mergeCell ref="A44:N44"/>
-    <mergeCell ref="K50:N50"/>
-    <mergeCell ref="K48:N48"/>
-    <mergeCell ref="A45:N45"/>
-    <mergeCell ref="C7:K7"/>
-    <mergeCell ref="C8:K8"/>
-    <mergeCell ref="A41:N41"/>
-    <mergeCell ref="K51:N51"/>
-    <mergeCell ref="K52:N52"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A3:N3"/>
     <mergeCell ref="A10:N10"/>
@@ -12059,6 +12051,24 @@
     <mergeCell ref="L20:M20"/>
     <mergeCell ref="D19:I19"/>
     <mergeCell ref="K38:L38"/>
+    <mergeCell ref="M79:M80"/>
+    <mergeCell ref="A59:N59"/>
+    <mergeCell ref="A61:N61"/>
+    <mergeCell ref="A42:N42"/>
+    <mergeCell ref="A44:N44"/>
+    <mergeCell ref="K50:N50"/>
+    <mergeCell ref="K48:N48"/>
+    <mergeCell ref="A45:N45"/>
+    <mergeCell ref="K51:N51"/>
+    <mergeCell ref="K52:N52"/>
+    <mergeCell ref="C5:K5"/>
+    <mergeCell ref="K37:L37"/>
+    <mergeCell ref="C6:K6"/>
+    <mergeCell ref="K79:K80"/>
+    <mergeCell ref="L79:L80"/>
+    <mergeCell ref="C7:K7"/>
+    <mergeCell ref="C8:K8"/>
+    <mergeCell ref="A41:N41"/>
   </mergeCells>
   <conditionalFormatting sqref="A30:A38">
     <cfRule type="cellIs" priority="1" stopIfTrue="1" operator="between">
@@ -12124,35 +12134,35 @@
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1">
       <c r="A2" s="387"/>
-      <c r="B2" s="660" t="s">
+      <c r="B2" s="649" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="660"/>
-      <c r="D2" s="660"/>
-      <c r="E2" s="660"/>
-      <c r="F2" s="660"/>
-      <c r="G2" s="660"/>
-      <c r="H2" s="660"/>
-      <c r="I2" s="660"/>
-      <c r="J2" s="660"/>
-      <c r="K2" s="660"/>
+      <c r="C2" s="649"/>
+      <c r="D2" s="649"/>
+      <c r="E2" s="649"/>
+      <c r="F2" s="649"/>
+      <c r="G2" s="649"/>
+      <c r="H2" s="649"/>
+      <c r="I2" s="649"/>
+      <c r="J2" s="649"/>
+      <c r="K2" s="649"/>
       <c r="L2" s="374"/>
       <c r="M2" s="386"/>
     </row>
     <row r="3" spans="1:14" ht="15" customHeight="1">
       <c r="A3" s="387"/>
-      <c r="B3" s="660" t="s">
+      <c r="B3" s="649" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="660"/>
-      <c r="D3" s="660"/>
-      <c r="E3" s="660"/>
-      <c r="F3" s="660"/>
-      <c r="G3" s="660"/>
-      <c r="H3" s="660"/>
-      <c r="I3" s="660"/>
-      <c r="J3" s="660"/>
-      <c r="K3" s="660"/>
+      <c r="C3" s="649"/>
+      <c r="D3" s="649"/>
+      <c r="E3" s="649"/>
+      <c r="F3" s="649"/>
+      <c r="G3" s="649"/>
+      <c r="H3" s="649"/>
+      <c r="I3" s="649"/>
+      <c r="J3" s="649"/>
+      <c r="K3" s="649"/>
       <c r="L3" s="374"/>
       <c r="M3" s="386"/>
     </row>
@@ -12173,12 +12183,12 @@
     </row>
     <row r="5" spans="1:14" ht="15" customHeight="1">
       <c r="A5" s="387"/>
-      <c r="B5" s="651" t="s">
+      <c r="B5" s="655" t="s">
         <v>126</v>
       </c>
-      <c r="C5" s="652"/>
-      <c r="D5" s="652"/>
-      <c r="E5" s="653"/>
+      <c r="C5" s="656"/>
+      <c r="D5" s="656"/>
+      <c r="E5" s="657"/>
       <c r="F5" s="331">
         <f>+Resumen!J26</f>
         <v>0</v>
@@ -12213,12 +12223,12 @@
     </row>
     <row r="7" spans="1:14" ht="15" customHeight="1">
       <c r="A7" s="387"/>
-      <c r="B7" s="651" t="s">
+      <c r="B7" s="655" t="s">
         <v>129</v>
       </c>
-      <c r="C7" s="652"/>
-      <c r="D7" s="652"/>
-      <c r="E7" s="653"/>
+      <c r="C7" s="656"/>
+      <c r="D7" s="656"/>
+      <c r="E7" s="657"/>
       <c r="F7" s="331">
         <f>+IF(F5="A",0.1,0.01)</f>
         <v>0.01</v>
@@ -12368,19 +12378,19 @@
       <c r="A17" s="396">
         <v>1</v>
       </c>
-      <c r="B17" s="654" t="s">
+      <c r="B17" s="658" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="655"/>
-      <c r="D17" s="655"/>
-      <c r="E17" s="656"/>
+      <c r="C17" s="659"/>
+      <c r="D17" s="659"/>
+      <c r="E17" s="660"/>
       <c r="F17" s="397" t="s">
         <v>36</v>
       </c>
       <c r="G17" s="426">
         <v>1</v>
       </c>
-      <c r="H17" s="662" t="s">
+      <c r="H17" s="651" t="s">
         <v>37</v>
       </c>
       <c r="J17" s="4" t="s">
@@ -12395,12 +12405,12 @@
       <c r="A18" s="396">
         <v>2</v>
       </c>
-      <c r="B18" s="654" t="s">
+      <c r="B18" s="658" t="s">
         <v>111</v>
       </c>
-      <c r="C18" s="655"/>
-      <c r="D18" s="655"/>
-      <c r="E18" s="656"/>
+      <c r="C18" s="659"/>
+      <c r="D18" s="659"/>
+      <c r="E18" s="660"/>
       <c r="F18" s="397" t="s">
         <v>36</v>
       </c>
@@ -12408,7 +12418,7 @@
         <f>+Resumen!I32</f>
         <v>0</v>
       </c>
-      <c r="H18" s="662"/>
+      <c r="H18" s="651"/>
       <c r="J18" s="4" t="s">
         <v>237</v>
       </c>
@@ -12421,12 +12431,12 @@
       <c r="A19" s="396">
         <v>3</v>
       </c>
-      <c r="B19" s="654" t="s">
+      <c r="B19" s="658" t="s">
         <v>112</v>
       </c>
-      <c r="C19" s="655"/>
-      <c r="D19" s="655"/>
-      <c r="E19" s="656"/>
+      <c r="C19" s="659"/>
+      <c r="D19" s="659"/>
+      <c r="E19" s="660"/>
       <c r="F19" s="397" t="s">
         <v>41</v>
       </c>
@@ -12450,12 +12460,12 @@
       <c r="A20" s="396">
         <v>4</v>
       </c>
-      <c r="B20" s="654" t="s">
+      <c r="B20" s="658" t="s">
         <v>113</v>
       </c>
-      <c r="C20" s="655"/>
-      <c r="D20" s="655"/>
-      <c r="E20" s="656"/>
+      <c r="C20" s="659"/>
+      <c r="D20" s="659"/>
+      <c r="E20" s="660"/>
       <c r="F20" s="397" t="s">
         <v>41</v>
       </c>
@@ -12508,12 +12518,12 @@
       <c r="A22" s="396">
         <v>6</v>
       </c>
-      <c r="B22" s="654" t="s">
+      <c r="B22" s="658" t="s">
         <v>114</v>
       </c>
-      <c r="C22" s="655"/>
-      <c r="D22" s="655"/>
-      <c r="E22" s="656"/>
+      <c r="C22" s="659"/>
+      <c r="D22" s="659"/>
+      <c r="E22" s="660"/>
       <c r="F22" s="399" t="s">
         <v>41</v>
       </c>
@@ -12537,12 +12547,12 @@
       <c r="A23" s="396">
         <v>7</v>
       </c>
-      <c r="B23" s="654" t="s">
+      <c r="B23" s="658" t="s">
         <v>115</v>
       </c>
-      <c r="C23" s="655"/>
-      <c r="D23" s="655"/>
-      <c r="E23" s="656"/>
+      <c r="C23" s="659"/>
+      <c r="D23" s="659"/>
+      <c r="E23" s="660"/>
       <c r="F23" s="397" t="s">
         <v>41</v>
       </c>
@@ -12566,12 +12576,12 @@
       <c r="A24" s="396">
         <v>8</v>
       </c>
-      <c r="B24" s="654" t="s">
+      <c r="B24" s="658" t="s">
         <v>116</v>
       </c>
-      <c r="C24" s="655"/>
-      <c r="D24" s="655"/>
-      <c r="E24" s="656"/>
+      <c r="C24" s="659"/>
+      <c r="D24" s="659"/>
+      <c r="E24" s="660"/>
       <c r="F24" s="399" t="s">
         <v>41</v>
       </c>
@@ -12595,12 +12605,12 @@
       <c r="A25" s="396">
         <v>9</v>
       </c>
-      <c r="B25" s="657" t="s">
+      <c r="B25" s="661" t="s">
         <v>117</v>
       </c>
-      <c r="C25" s="658"/>
-      <c r="D25" s="658"/>
-      <c r="E25" s="659"/>
+      <c r="C25" s="662"/>
+      <c r="D25" s="662"/>
+      <c r="E25" s="663"/>
       <c r="F25" s="399" t="s">
         <v>56</v>
       </c>
@@ -12716,24 +12726,24 @@
     </row>
     <row r="31" spans="1:12" ht="15.9" customHeight="1">
       <c r="A31" s="387"/>
-      <c r="B31" s="661" t="s">
+      <c r="B31" s="650" t="s">
         <v>137</v>
       </c>
-      <c r="C31" s="661"/>
-      <c r="D31" s="661"/>
-      <c r="E31" s="661"/>
-      <c r="F31" s="661"/>
-      <c r="G31" s="661"/>
+      <c r="C31" s="650"/>
+      <c r="D31" s="650"/>
+      <c r="E31" s="650"/>
+      <c r="F31" s="650"/>
+      <c r="G31" s="650"/>
       <c r="L31" s="394"/>
     </row>
     <row r="32" spans="1:12" ht="26.25" customHeight="1">
       <c r="A32" s="387"/>
-      <c r="B32" s="651" t="s">
+      <c r="B32" s="655" t="s">
         <v>138</v>
       </c>
-      <c r="C32" s="652"/>
-      <c r="D32" s="652"/>
-      <c r="E32" s="653"/>
+      <c r="C32" s="656"/>
+      <c r="D32" s="656"/>
+      <c r="E32" s="657"/>
       <c r="F32" s="369" t="s">
         <v>139</v>
       </c>
@@ -12744,12 +12754,12 @@
     </row>
     <row r="33" spans="1:12" ht="16.5" customHeight="1">
       <c r="A33" s="387"/>
-      <c r="B33" s="648" t="s">
+      <c r="B33" s="652" t="s">
         <v>141</v>
       </c>
-      <c r="C33" s="649"/>
-      <c r="D33" s="649"/>
-      <c r="E33" s="650"/>
+      <c r="C33" s="653"/>
+      <c r="D33" s="653"/>
+      <c r="E33" s="654"/>
       <c r="F33" s="330" t="s">
         <v>142</v>
       </c>
@@ -12760,12 +12770,12 @@
     </row>
     <row r="34" spans="1:12" ht="16.5" customHeight="1">
       <c r="A34" s="387"/>
-      <c r="B34" s="648" t="s">
+      <c r="B34" s="652" t="s">
         <v>143</v>
       </c>
-      <c r="C34" s="649"/>
-      <c r="D34" s="649"/>
-      <c r="E34" s="650"/>
+      <c r="C34" s="653"/>
+      <c r="D34" s="653"/>
+      <c r="E34" s="654"/>
       <c r="F34" s="330" t="s">
         <v>144</v>
       </c>
@@ -12776,12 +12786,12 @@
     </row>
     <row r="35" spans="1:12" ht="16.5" customHeight="1">
       <c r="A35" s="387"/>
-      <c r="B35" s="648" t="s">
+      <c r="B35" s="652" t="s">
         <v>145</v>
       </c>
-      <c r="C35" s="649"/>
-      <c r="D35" s="649"/>
-      <c r="E35" s="650"/>
+      <c r="C35" s="653"/>
+      <c r="D35" s="653"/>
+      <c r="E35" s="654"/>
       <c r="F35" s="330" t="s">
         <v>146</v>
       </c>
@@ -12792,24 +12802,24 @@
     </row>
     <row r="36" spans="1:12" ht="16.5" customHeight="1">
       <c r="A36" s="387"/>
-      <c r="B36" s="661" t="s">
+      <c r="B36" s="650" t="s">
         <v>147</v>
       </c>
-      <c r="C36" s="661"/>
-      <c r="D36" s="661"/>
-      <c r="E36" s="661"/>
-      <c r="F36" s="661"/>
-      <c r="G36" s="661"/>
+      <c r="C36" s="650"/>
+      <c r="D36" s="650"/>
+      <c r="E36" s="650"/>
+      <c r="F36" s="650"/>
+      <c r="G36" s="650"/>
       <c r="L36" s="394"/>
     </row>
     <row r="37" spans="1:12" ht="16.5" customHeight="1">
       <c r="A37" s="387"/>
-      <c r="B37" s="648" t="s">
+      <c r="B37" s="652" t="s">
         <v>227</v>
       </c>
-      <c r="C37" s="649"/>
-      <c r="D37" s="649"/>
-      <c r="E37" s="650"/>
+      <c r="C37" s="653"/>
+      <c r="D37" s="653"/>
+      <c r="E37" s="654"/>
       <c r="F37" s="330" t="s">
         <v>148</v>
       </c>
@@ -12820,12 +12830,12 @@
     </row>
     <row r="38" spans="1:12" ht="16.5" customHeight="1">
       <c r="A38" s="387"/>
-      <c r="B38" s="648" t="s">
+      <c r="B38" s="652" t="s">
         <v>149</v>
       </c>
-      <c r="C38" s="649"/>
-      <c r="D38" s="649"/>
-      <c r="E38" s="650"/>
+      <c r="C38" s="653"/>
+      <c r="D38" s="653"/>
+      <c r="E38" s="654"/>
       <c r="F38" s="330" t="s">
         <v>150</v>
       </c>
@@ -12836,12 +12846,12 @@
     </row>
     <row r="39" spans="1:12" ht="16.5" customHeight="1">
       <c r="A39" s="387"/>
-      <c r="B39" s="648" t="s">
+      <c r="B39" s="652" t="s">
         <v>151</v>
       </c>
-      <c r="C39" s="649"/>
-      <c r="D39" s="649"/>
-      <c r="E39" s="650"/>
+      <c r="C39" s="653"/>
+      <c r="D39" s="653"/>
+      <c r="E39" s="654"/>
       <c r="F39" s="330" t="s">
         <v>152</v>
       </c>
@@ -12957,15 +12967,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="B31:G31"/>
-    <mergeCell ref="B36:G36"/>
-    <mergeCell ref="H17:H18"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B34:E34"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B32:E32"/>
     <mergeCell ref="B39:E39"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B7:E7"/>
@@ -12979,6 +12980,15 @@
     <mergeCell ref="B25:E25"/>
     <mergeCell ref="B37:E37"/>
     <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="H17:H18"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B32:E32"/>
   </mergeCells>
   <conditionalFormatting sqref="E11">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="no">
@@ -13023,16 +13033,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="12.75" customHeight="1">
-      <c r="A1" s="672"/>
-      <c r="B1" s="673"/>
-      <c r="C1" s="663" t="s">
+      <c r="A1" s="681"/>
+      <c r="B1" s="682"/>
+      <c r="C1" s="672" t="s">
         <v>153</v>
       </c>
-      <c r="D1" s="664"/>
-      <c r="E1" s="664"/>
-      <c r="F1" s="664"/>
-      <c r="G1" s="664"/>
-      <c r="H1" s="665"/>
+      <c r="D1" s="673"/>
+      <c r="E1" s="673"/>
+      <c r="F1" s="673"/>
+      <c r="G1" s="673"/>
+      <c r="H1" s="674"/>
       <c r="I1" s="221" t="s">
         <v>154</v>
       </c>
@@ -13041,14 +13051,14 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="12.75" customHeight="1">
-      <c r="A2" s="674"/>
-      <c r="B2" s="675"/>
-      <c r="C2" s="666"/>
-      <c r="D2" s="667"/>
-      <c r="E2" s="667"/>
-      <c r="F2" s="667"/>
-      <c r="G2" s="667"/>
-      <c r="H2" s="668"/>
+      <c r="A2" s="683"/>
+      <c r="B2" s="684"/>
+      <c r="C2" s="675"/>
+      <c r="D2" s="676"/>
+      <c r="E2" s="676"/>
+      <c r="F2" s="676"/>
+      <c r="G2" s="676"/>
+      <c r="H2" s="677"/>
       <c r="I2" s="221" t="s">
         <v>156</v>
       </c>
@@ -13057,14 +13067,14 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="12.75" customHeight="1">
-      <c r="A3" s="674"/>
-      <c r="B3" s="675"/>
-      <c r="C3" s="666"/>
-      <c r="D3" s="667"/>
-      <c r="E3" s="667"/>
-      <c r="F3" s="667"/>
-      <c r="G3" s="667"/>
-      <c r="H3" s="668"/>
+      <c r="A3" s="683"/>
+      <c r="B3" s="684"/>
+      <c r="C3" s="675"/>
+      <c r="D3" s="676"/>
+      <c r="E3" s="676"/>
+      <c r="F3" s="676"/>
+      <c r="G3" s="676"/>
+      <c r="H3" s="677"/>
       <c r="I3" s="221" t="s">
         <v>157</v>
       </c>
@@ -13073,14 +13083,14 @@
       </c>
     </row>
     <row r="4" spans="1:10" ht="12.75" customHeight="1">
-      <c r="A4" s="676"/>
-      <c r="B4" s="677"/>
-      <c r="C4" s="669"/>
-      <c r="D4" s="670"/>
-      <c r="E4" s="670"/>
-      <c r="F4" s="670"/>
-      <c r="G4" s="670"/>
-      <c r="H4" s="671"/>
+      <c r="A4" s="685"/>
+      <c r="B4" s="686"/>
+      <c r="C4" s="678"/>
+      <c r="D4" s="679"/>
+      <c r="E4" s="679"/>
+      <c r="F4" s="679"/>
+      <c r="G4" s="679"/>
+      <c r="H4" s="680"/>
       <c r="I4" s="221" t="s">
         <v>158</v>
       </c>
@@ -13227,16 +13237,16 @@
       <c r="J37" s="337"/>
     </row>
     <row r="38" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A38" s="682" t="s">
+      <c r="A38" s="691" t="s">
         <v>304</v>
       </c>
-      <c r="B38" s="683"/>
-      <c r="C38" s="683"/>
-      <c r="D38" s="683"/>
-      <c r="E38" s="683"/>
-      <c r="F38" s="683"/>
-      <c r="G38" s="683"/>
-      <c r="H38" s="684"/>
+      <c r="B38" s="692"/>
+      <c r="C38" s="692"/>
+      <c r="D38" s="692"/>
+      <c r="E38" s="692"/>
+      <c r="F38" s="692"/>
+      <c r="G38" s="692"/>
+      <c r="H38" s="693"/>
       <c r="I38" s="337"/>
       <c r="J38" s="337"/>
     </row>
@@ -13670,42 +13680,42 @@
       <c r="J53" s="337"/>
     </row>
     <row r="54" spans="1:10" s="343" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A54" s="685" t="s">
+      <c r="A54" s="694" t="s">
         <v>195</v>
       </c>
-      <c r="B54" s="686"/>
-      <c r="C54" s="687"/>
+      <c r="B54" s="695"/>
+      <c r="C54" s="696"/>
       <c r="D54" s="280" t="s">
         <v>56</v>
       </c>
       <c r="E54" s="281"/>
-      <c r="F54" s="678" t="e">
+      <c r="F54" s="687" t="e">
         <f>SQRT((H41*H41)+(H45*H45)+(H49*H49)+(H53*H53))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="G54" s="678"/>
-      <c r="H54" s="679"/>
+      <c r="G54" s="687"/>
+      <c r="H54" s="688"/>
       <c r="I54" s="337" t="s">
         <v>196</v>
       </c>
       <c r="J54" s="337"/>
     </row>
     <row r="55" spans="1:10" s="343" customFormat="1" ht="18" customHeight="1" thickBot="1">
-      <c r="A55" s="688" t="s">
+      <c r="A55" s="697" t="s">
         <v>197</v>
       </c>
-      <c r="B55" s="689"/>
-      <c r="C55" s="690"/>
+      <c r="B55" s="698"/>
+      <c r="C55" s="699"/>
       <c r="D55" s="308" t="s">
         <v>56</v>
       </c>
       <c r="E55" s="282"/>
-      <c r="F55" s="680" t="e">
+      <c r="F55" s="689" t="e">
         <f>F54*2</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="G55" s="680"/>
-      <c r="H55" s="681"/>
+      <c r="G55" s="689"/>
+      <c r="H55" s="690"/>
       <c r="I55" s="337" t="s">
         <v>198</v>
       </c>
@@ -13878,46 +13888,40 @@
       <c r="A70" s="541" t="s">
         <v>306</v>
       </c>
-      <c r="B70" s="691" t="s">
+      <c r="B70" s="664" t="s">
         <v>307</v>
       </c>
-      <c r="C70" s="692"/>
+      <c r="C70" s="665"/>
       <c r="D70" s="542"/>
-      <c r="E70" s="693" t="s">
+      <c r="E70" s="666" t="s">
         <v>308</v>
       </c>
-      <c r="F70" s="693"/>
-      <c r="G70" s="694" t="s">
+      <c r="F70" s="666"/>
+      <c r="G70" s="667" t="s">
         <v>309</v>
       </c>
-      <c r="H70" s="695"/>
+      <c r="H70" s="668"/>
     </row>
     <row r="72" spans="1:10">
       <c r="A72" s="543" t="s">
         <v>310</v>
       </c>
-      <c r="B72" s="696">
+      <c r="B72" s="669">
         <v>44944</v>
       </c>
-      <c r="C72" s="697"/>
-      <c r="E72" s="698" t="s">
+      <c r="C72" s="670"/>
+      <c r="E72" s="671" t="s">
         <v>311</v>
       </c>
-      <c r="F72" s="698"/>
-      <c r="G72" s="696">
+      <c r="F72" s="671"/>
+      <c r="G72" s="669">
         <v>44944</v>
       </c>
-      <c r="H72" s="697"/>
+      <c r="H72" s="670"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="iLEnVB6pm8HGxp/myiIucvHcjmqcSrUFV5EFJhRy/Wl6J20Lu8rufg9gJo4vTQR/wN6I3HZ06PN9TnsphGZBRg==" saltValue="rC1uvtCaR6F4sqhd68ayKA==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="13">
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="E70:F70"/>
-    <mergeCell ref="G70:H70"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="E72:F72"/>
-    <mergeCell ref="G72:H72"/>
     <mergeCell ref="C1:H4"/>
     <mergeCell ref="A1:B4"/>
     <mergeCell ref="F54:H54"/>
@@ -13925,6 +13929,12 @@
     <mergeCell ref="A38:H38"/>
     <mergeCell ref="A54:C54"/>
     <mergeCell ref="A55:C55"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="E70:F70"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="E72:F72"/>
+    <mergeCell ref="G72:H72"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.31496062992125984" top="0.74803149606299213" bottom="0.55118110236220474" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="70" orientation="portrait" r:id="rId1"/>
@@ -14227,22 +14237,22 @@
       </c>
     </row>
     <row r="18" spans="3:15">
-      <c r="C18" s="699" t="s">
+      <c r="C18" s="700" t="s">
         <v>209</v>
       </c>
-      <c r="D18" s="699"/>
-      <c r="E18" s="699"/>
-      <c r="F18" s="699"/>
-      <c r="G18" s="699"/>
-      <c r="H18" s="699"/>
-      <c r="J18" s="701" t="s">
+      <c r="D18" s="700"/>
+      <c r="E18" s="700"/>
+      <c r="F18" s="700"/>
+      <c r="G18" s="700"/>
+      <c r="H18" s="700"/>
+      <c r="J18" s="702" t="s">
         <v>209</v>
       </c>
-      <c r="K18" s="702"/>
-      <c r="L18" s="702"/>
-      <c r="M18" s="702"/>
-      <c r="N18" s="702"/>
-      <c r="O18" s="703"/>
+      <c r="K18" s="703"/>
+      <c r="L18" s="703"/>
+      <c r="M18" s="703"/>
+      <c r="N18" s="703"/>
+      <c r="O18" s="704"/>
     </row>
     <row r="19" spans="3:15">
       <c r="C19" s="213"/>
@@ -14252,9 +14262,9 @@
       <c r="G19" s="214"/>
       <c r="H19" s="215"/>
       <c r="J19" s="263"/>
-      <c r="K19" s="700"/>
-      <c r="L19" s="700"/>
-      <c r="M19" s="700"/>
+      <c r="K19" s="701"/>
+      <c r="L19" s="701"/>
+      <c r="M19" s="701"/>
       <c r="N19" s="214"/>
       <c r="O19" s="215"/>
     </row>
@@ -14503,22 +14513,22 @@
       <c r="B7" s="283" t="s">
         <v>210</v>
       </c>
-      <c r="C7" s="704">
+      <c r="C7" s="705">
         <v>0.11832159566199267</v>
       </c>
-      <c r="D7" s="704"/>
-      <c r="E7" s="704"/>
+      <c r="D7" s="705"/>
+      <c r="E7" s="705"/>
       <c r="F7" s="284"/>
     </row>
     <row r="8" spans="2:6" ht="15" customHeight="1">
       <c r="B8" s="283" t="s">
         <v>211</v>
       </c>
-      <c r="C8" s="704">
+      <c r="C8" s="705">
         <v>0.11937336386339086</v>
       </c>
-      <c r="D8" s="704"/>
-      <c r="E8" s="704"/>
+      <c r="D8" s="705"/>
+      <c r="E8" s="705"/>
       <c r="F8" s="284"/>
     </row>
     <row r="9" spans="2:6" ht="15" customHeight="1"/>
@@ -14552,10 +14562,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="18.75" customHeight="1">
-      <c r="A2" s="705" t="s">
+      <c r="A2" s="706" t="s">
         <v>212</v>
       </c>
-      <c r="B2" s="705"/>
+      <c r="B2" s="706"/>
       <c r="C2" s="5" t="s">
         <v>213</v>
       </c>

</xml_diff>